<commit_message>
feat: add municipal European ESB tender ArchiMate model
42 elements across 3 layers, 51 relationships, 3 scoped views:
- Full Architecture View (all 42 elements)
- Tender Process (20 business elements, EU phases 1-9)
- ESB Solution Architecture (13 app + 9 tech elements)

Also fixes view scoping in generate_model.py (Include Elements column header match)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/model-input.xlsx
+++ b/model-input.xlsx
@@ -124,7 +124,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -180,6 +180,21 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -948,284 +963,664 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="10" t="inlineStr"/>
-      <c r="B2" s="10" t="inlineStr">
-        <is>
-          <t>Customer</t>
-        </is>
-      </c>
-      <c r="C2" s="10" t="inlineStr">
+      <c r="A2" s="20" t="inlineStr">
+        <is>
+          <t>b001</t>
+        </is>
+      </c>
+      <c r="B2" s="20" t="inlineStr">
+        <is>
+          <t>Municipality</t>
+        </is>
+      </c>
+      <c r="C2" s="20" t="inlineStr">
         <is>
           <t>BusinessActor</t>
         </is>
       </c>
       <c r="D2" s="11" t="inlineStr">
         <is>
-          <t>End user interacting with the platform</t>
+          <t>Contracting authority issuing the ESB tender under EU Directive 2014/24/EU</t>
         </is>
       </c>
       <c r="E2" s="11" t="inlineStr"/>
-      <c r="F2" s="10" t="inlineStr">
-        <is>
-          <t>core, external</t>
-        </is>
-      </c>
-      <c r="G2" s="10" t="inlineStr">
+      <c r="F2" s="20" t="inlineStr">
+        <is>
+          <t>contracting-authority</t>
+        </is>
+      </c>
+      <c r="G2" s="20" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="10" t="inlineStr"/>
-      <c r="B3" s="10" t="inlineStr">
-        <is>
-          <t>Account Manager</t>
-        </is>
-      </c>
-      <c r="C3" s="10" t="inlineStr">
+      <c r="A3" s="20" t="inlineStr">
+        <is>
+          <t>b002</t>
+        </is>
+      </c>
+      <c r="B3" s="20" t="inlineStr">
+        <is>
+          <t>ESB Vendor</t>
+        </is>
+      </c>
+      <c r="C3" s="20" t="inlineStr">
+        <is>
+          <t>BusinessActor</t>
+        </is>
+      </c>
+      <c r="D3" s="11" t="inlineStr">
+        <is>
+          <t>Supplier submitting a tender offer for the ESB solution</t>
+        </is>
+      </c>
+      <c r="E3" s="11" t="inlineStr"/>
+      <c r="F3" s="20" t="inlineStr">
+        <is>
+          <t>vendor, tenderer</t>
+        </is>
+      </c>
+      <c r="G3" s="20" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="20" t="inlineStr">
+        <is>
+          <t>b003</t>
+        </is>
+      </c>
+      <c r="B4" s="20" t="inlineStr">
+        <is>
+          <t>Evaluation Committee</t>
+        </is>
+      </c>
+      <c r="C4" s="20" t="inlineStr">
+        <is>
+          <t>BusinessCollaboration</t>
+        </is>
+      </c>
+      <c r="D4" s="11" t="inlineStr">
+        <is>
+          <t>Multi-disciplinary team assessing offers on technical and financial criteria</t>
+        </is>
+      </c>
+      <c r="E4" s="11" t="inlineStr"/>
+      <c r="F4" s="20" t="inlineStr">
+        <is>
+          <t>procurement, evaluation</t>
+        </is>
+      </c>
+      <c r="G4" s="20" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="20" t="inlineStr">
+        <is>
+          <t>b004</t>
+        </is>
+      </c>
+      <c r="B5" s="20" t="inlineStr">
+        <is>
+          <t>Contracting Officer</t>
+        </is>
+      </c>
+      <c r="C5" s="20" t="inlineStr">
         <is>
           <t>BusinessRole</t>
         </is>
       </c>
-      <c r="D3" s="11" t="inlineStr">
-        <is>
-          <t>Internal role managing customer accounts</t>
-        </is>
-      </c>
-      <c r="E3" s="11" t="inlineStr"/>
-      <c r="F3" s="10" t="inlineStr">
-        <is>
-          <t>internal</t>
-        </is>
-      </c>
-      <c r="G3" s="10" t="inlineStr">
+      <c r="D5" s="11" t="inlineStr">
+        <is>
+          <t>Manages the full procurement process and ensures legal compliance</t>
+        </is>
+      </c>
+      <c r="E5" s="11" t="inlineStr"/>
+      <c r="F5" s="20" t="inlineStr">
+        <is>
+          <t>procurement</t>
+        </is>
+      </c>
+      <c r="G5" s="20" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="10" t="inlineStr"/>
-      <c r="B4" s="10" t="inlineStr">
-        <is>
-          <t>Order Management</t>
-        </is>
-      </c>
-      <c r="C4" s="10" t="inlineStr">
+    <row r="6">
+      <c r="A6" s="20" t="inlineStr">
+        <is>
+          <t>b005</t>
+        </is>
+      </c>
+      <c r="B6" s="20" t="inlineStr">
+        <is>
+          <t>IT Architect</t>
+        </is>
+      </c>
+      <c r="C6" s="20" t="inlineStr">
+        <is>
+          <t>BusinessRole</t>
+        </is>
+      </c>
+      <c r="D6" s="11" t="inlineStr">
+        <is>
+          <t>Defines technical requirements and assesses vendor solutions</t>
+        </is>
+      </c>
+      <c r="E6" s="11" t="inlineStr"/>
+      <c r="F6" s="20" t="inlineStr">
+        <is>
+          <t>technical</t>
+        </is>
+      </c>
+      <c r="G6" s="20" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="20" t="inlineStr">
+        <is>
+          <t>b006</t>
+        </is>
+      </c>
+      <c r="B7" s="20" t="inlineStr">
+        <is>
+          <t>Legal Advisor</t>
+        </is>
+      </c>
+      <c r="C7" s="20" t="inlineStr">
+        <is>
+          <t>BusinessRole</t>
+        </is>
+      </c>
+      <c r="D7" s="11" t="inlineStr">
+        <is>
+          <t>Ensures tender process complies with EU and national procurement law</t>
+        </is>
+      </c>
+      <c r="E7" s="11" t="inlineStr"/>
+      <c r="F7" s="20" t="inlineStr">
+        <is>
+          <t>legal, compliance</t>
+        </is>
+      </c>
+      <c r="G7" s="20" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="20" t="inlineStr">
+        <is>
+          <t>b007</t>
+        </is>
+      </c>
+      <c r="B8" s="20" t="inlineStr">
+        <is>
+          <t>Needs Assessment</t>
+        </is>
+      </c>
+      <c r="C8" s="20" t="inlineStr">
         <is>
           <t>BusinessProcess</t>
         </is>
       </c>
-      <c r="D4" s="11" t="inlineStr">
-        <is>
-          <t>Process for handling customer orders end-to-end</t>
-        </is>
-      </c>
-      <c r="E4" s="11" t="inlineStr"/>
-      <c r="F4" s="10" t="inlineStr">
-        <is>
-          <t>core</t>
-        </is>
-      </c>
-      <c r="G4" s="10" t="inlineStr">
+      <c r="D8" s="11" t="inlineStr">
+        <is>
+          <t>Identify functional and non-functional ESB requirements across the municipality</t>
+        </is>
+      </c>
+      <c r="E8" s="11" t="inlineStr"/>
+      <c r="F8" s="20" t="inlineStr">
+        <is>
+          <t>phase-1</t>
+        </is>
+      </c>
+      <c r="G8" s="20" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="10" t="inlineStr"/>
-      <c r="B5" s="10" t="inlineStr">
-        <is>
-          <t>Product Catalog Service</t>
-        </is>
-      </c>
-      <c r="C5" s="10" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="20" t="inlineStr">
+        <is>
+          <t>b008</t>
+        </is>
+      </c>
+      <c r="B9" s="20" t="inlineStr">
+        <is>
+          <t>Market Consultation</t>
+        </is>
+      </c>
+      <c r="C9" s="20" t="inlineStr">
+        <is>
+          <t>BusinessProcess</t>
+        </is>
+      </c>
+      <c r="D9" s="11" t="inlineStr">
+        <is>
+          <t>Prior Information Notice (PIN) and Request for Information to map the ESB market</t>
+        </is>
+      </c>
+      <c r="E9" s="11" t="inlineStr"/>
+      <c r="F9" s="20" t="inlineStr">
+        <is>
+          <t>phase-2</t>
+        </is>
+      </c>
+      <c r="G9" s="20" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="20" t="inlineStr">
+        <is>
+          <t>b009</t>
+        </is>
+      </c>
+      <c r="B10" s="20" t="inlineStr">
+        <is>
+          <t>Tender Preparation</t>
+        </is>
+      </c>
+      <c r="C10" s="20" t="inlineStr">
+        <is>
+          <t>BusinessProcess</t>
+        </is>
+      </c>
+      <c r="D10" s="11" t="inlineStr">
+        <is>
+          <t>Draft technical specifications, award criteria, and tender documents per EU rules</t>
+        </is>
+      </c>
+      <c r="E10" s="11" t="inlineStr"/>
+      <c r="F10" s="20" t="inlineStr">
+        <is>
+          <t>phase-3</t>
+        </is>
+      </c>
+      <c r="G10" s="20" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="20" t="inlineStr">
+        <is>
+          <t>b010</t>
+        </is>
+      </c>
+      <c r="B11" s="20" t="inlineStr">
+        <is>
+          <t>Tender Publication</t>
+        </is>
+      </c>
+      <c r="C11" s="20" t="inlineStr">
+        <is>
+          <t>BusinessProcess</t>
+        </is>
+      </c>
+      <c r="D11" s="11" t="inlineStr">
+        <is>
+          <t>Publish call for tender on TED (Tenders Electronic Daily) and national platform</t>
+        </is>
+      </c>
+      <c r="E11" s="11" t="inlineStr"/>
+      <c r="F11" s="20" t="inlineStr">
+        <is>
+          <t>phase-4</t>
+        </is>
+      </c>
+      <c r="G11" s="20" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="20" t="inlineStr">
+        <is>
+          <t>b011</t>
+        </is>
+      </c>
+      <c r="B12" s="20" t="inlineStr">
+        <is>
+          <t>Tender Reception</t>
+        </is>
+      </c>
+      <c r="C12" s="20" t="inlineStr">
+        <is>
+          <t>BusinessProcess</t>
+        </is>
+      </c>
+      <c r="D12" s="11" t="inlineStr">
+        <is>
+          <t>Receive, register and safeguard vendor offers within the submission deadline</t>
+        </is>
+      </c>
+      <c r="E12" s="11" t="inlineStr"/>
+      <c r="F12" s="20" t="inlineStr">
+        <is>
+          <t>phase-5</t>
+        </is>
+      </c>
+      <c r="G12" s="20" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="20" t="inlineStr">
+        <is>
+          <t>b012</t>
+        </is>
+      </c>
+      <c r="B13" s="20" t="inlineStr">
+        <is>
+          <t>Tender Evaluation</t>
+        </is>
+      </c>
+      <c r="C13" s="20" t="inlineStr">
+        <is>
+          <t>BusinessProcess</t>
+        </is>
+      </c>
+      <c r="D13" s="11" t="inlineStr">
+        <is>
+          <t>Assess offers against technical (BPQR) and financial criteria; MEAT principle</t>
+        </is>
+      </c>
+      <c r="E13" s="11" t="inlineStr"/>
+      <c r="F13" s="20" t="inlineStr">
+        <is>
+          <t>phase-6</t>
+        </is>
+      </c>
+      <c r="G13" s="20" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="20" t="inlineStr">
+        <is>
+          <t>b013</t>
+        </is>
+      </c>
+      <c r="B14" s="20" t="inlineStr">
+        <is>
+          <t>Contract Award</t>
+        </is>
+      </c>
+      <c r="C14" s="20" t="inlineStr">
+        <is>
+          <t>BusinessProcess</t>
+        </is>
+      </c>
+      <c r="D14" s="11" t="inlineStr">
+        <is>
+          <t>Notify winning vendor, publish award notice on TED, observe standstill period</t>
+        </is>
+      </c>
+      <c r="E14" s="11" t="inlineStr"/>
+      <c r="F14" s="20" t="inlineStr">
+        <is>
+          <t>phase-7</t>
+        </is>
+      </c>
+      <c r="G14" s="20" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="20" t="inlineStr">
+        <is>
+          <t>b014</t>
+        </is>
+      </c>
+      <c r="B15" s="20" t="inlineStr">
+        <is>
+          <t>ESB Implementation</t>
+        </is>
+      </c>
+      <c r="C15" s="20" t="inlineStr">
+        <is>
+          <t>BusinessProcess</t>
+        </is>
+      </c>
+      <c r="D15" s="11" t="inlineStr">
+        <is>
+          <t>Deploy, configure and integrate the ESB solution within municipal IT landscape</t>
+        </is>
+      </c>
+      <c r="E15" s="11" t="inlineStr"/>
+      <c r="F15" s="20" t="inlineStr">
+        <is>
+          <t>phase-8</t>
+        </is>
+      </c>
+      <c r="G15" s="20" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="20" t="inlineStr">
+        <is>
+          <t>b015</t>
+        </is>
+      </c>
+      <c r="B16" s="20" t="inlineStr">
+        <is>
+          <t>Acceptance Testing</t>
+        </is>
+      </c>
+      <c r="C16" s="20" t="inlineStr">
+        <is>
+          <t>BusinessProcess</t>
+        </is>
+      </c>
+      <c r="D16" s="11" t="inlineStr">
+        <is>
+          <t>Formal acceptance test and go-live sign-off by municipal IT and business owners</t>
+        </is>
+      </c>
+      <c r="E16" s="11" t="inlineStr"/>
+      <c r="F16" s="20" t="inlineStr">
+        <is>
+          <t>phase-9</t>
+        </is>
+      </c>
+      <c r="G16" s="20" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="20" t="inlineStr">
+        <is>
+          <t>b016</t>
+        </is>
+      </c>
+      <c r="B17" s="20" t="inlineStr">
+        <is>
+          <t>Procurement Service</t>
+        </is>
+      </c>
+      <c r="C17" s="20" t="inlineStr">
         <is>
           <t>BusinessService</t>
         </is>
       </c>
-      <c r="D5" s="11" t="inlineStr">
-        <is>
-          <t>Provides product information to customers</t>
-        </is>
-      </c>
-      <c r="E5" s="11" t="inlineStr"/>
-      <c r="F5" s="10" t="inlineStr">
-        <is>
-          <t>core</t>
-        </is>
-      </c>
-      <c r="G5" s="10" t="inlineStr">
+      <c r="D17" s="11" t="inlineStr">
+        <is>
+          <t>End-to-end procurement management service provided to the municipality</t>
+        </is>
+      </c>
+      <c r="E17" s="11" t="inlineStr"/>
+      <c r="F17" s="20" t="inlineStr">
+        <is>
+          <t>service</t>
+        </is>
+      </c>
+      <c r="G17" s="20" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="10" t="inlineStr"/>
-      <c r="B6" s="10" t="inlineStr">
-        <is>
-          <t>Order</t>
-        </is>
-      </c>
-      <c r="C6" s="10" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="20" t="inlineStr">
+        <is>
+          <t>b017</t>
+        </is>
+      </c>
+      <c r="B18" s="20" t="inlineStr">
+        <is>
+          <t>Technical Spec</t>
+        </is>
+      </c>
+      <c r="C18" s="20" t="inlineStr">
         <is>
           <t>BusinessObject</t>
         </is>
       </c>
-      <c r="D6" s="11" t="inlineStr">
-        <is>
-          <t>Represents a customer order</t>
-        </is>
-      </c>
-      <c r="E6" s="11" t="inlineStr"/>
-      <c r="F6" s="10" t="inlineStr">
-        <is>
-          <t>data</t>
-        </is>
-      </c>
-      <c r="G6" s="10" t="inlineStr">
+      <c r="D18" s="11" t="inlineStr">
+        <is>
+          <t>Document defining ESB functional requirements, integration scenarios and NFRs</t>
+        </is>
+      </c>
+      <c r="E18" s="11" t="inlineStr"/>
+      <c r="F18" s="20" t="inlineStr">
+        <is>
+          <t>document</t>
+        </is>
+      </c>
+      <c r="G18" s="20" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="10" t="n"/>
-      <c r="B7" s="10" t="n"/>
-      <c r="C7" s="10" t="n"/>
-      <c r="D7" s="11" t="n"/>
-      <c r="E7" s="11" t="n"/>
-      <c r="F7" s="10" t="n"/>
-      <c r="G7" s="10" t="n"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="10" t="n"/>
-      <c r="B8" s="10" t="n"/>
-      <c r="C8" s="10" t="n"/>
-      <c r="D8" s="11" t="n"/>
-      <c r="E8" s="11" t="n"/>
-      <c r="F8" s="10" t="n"/>
-      <c r="G8" s="10" t="n"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="10" t="n"/>
-      <c r="B9" s="10" t="n"/>
-      <c r="C9" s="10" t="n"/>
-      <c r="D9" s="11" t="n"/>
-      <c r="E9" s="11" t="n"/>
-      <c r="F9" s="10" t="n"/>
-      <c r="G9" s="10" t="n"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="10" t="n"/>
-      <c r="B10" s="10" t="n"/>
-      <c r="C10" s="10" t="n"/>
-      <c r="D10" s="11" t="n"/>
-      <c r="E10" s="11" t="n"/>
-      <c r="F10" s="10" t="n"/>
-      <c r="G10" s="10" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="10" t="n"/>
-      <c r="B11" s="10" t="n"/>
-      <c r="C11" s="10" t="n"/>
-      <c r="D11" s="11" t="n"/>
-      <c r="E11" s="11" t="n"/>
-      <c r="F11" s="10" t="n"/>
-      <c r="G11" s="10" t="n"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="10" t="n"/>
-      <c r="B12" s="10" t="n"/>
-      <c r="C12" s="10" t="n"/>
-      <c r="D12" s="11" t="n"/>
-      <c r="E12" s="11" t="n"/>
-      <c r="F12" s="10" t="n"/>
-      <c r="G12" s="10" t="n"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="10" t="n"/>
-      <c r="B13" s="10" t="n"/>
-      <c r="C13" s="10" t="n"/>
-      <c r="D13" s="11" t="n"/>
-      <c r="E13" s="11" t="n"/>
-      <c r="F13" s="10" t="n"/>
-      <c r="G13" s="10" t="n"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="10" t="n"/>
-      <c r="B14" s="10" t="n"/>
-      <c r="C14" s="10" t="n"/>
-      <c r="D14" s="11" t="n"/>
-      <c r="E14" s="11" t="n"/>
-      <c r="F14" s="10" t="n"/>
-      <c r="G14" s="10" t="n"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="10" t="n"/>
-      <c r="B15" s="10" t="n"/>
-      <c r="C15" s="10" t="n"/>
-      <c r="D15" s="11" t="n"/>
-      <c r="E15" s="11" t="n"/>
-      <c r="F15" s="10" t="n"/>
-      <c r="G15" s="10" t="n"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="10" t="n"/>
-      <c r="B16" s="10" t="n"/>
-      <c r="C16" s="10" t="n"/>
-      <c r="D16" s="11" t="n"/>
-      <c r="E16" s="11" t="n"/>
-      <c r="F16" s="10" t="n"/>
-      <c r="G16" s="10" t="n"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="10" t="n"/>
-      <c r="B17" s="10" t="n"/>
-      <c r="C17" s="10" t="n"/>
-      <c r="D17" s="11" t="n"/>
-      <c r="E17" s="11" t="n"/>
-      <c r="F17" s="10" t="n"/>
-      <c r="G17" s="10" t="n"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="10" t="n"/>
-      <c r="B18" s="10" t="n"/>
-      <c r="C18" s="10" t="n"/>
-      <c r="D18" s="11" t="n"/>
-      <c r="E18" s="11" t="n"/>
-      <c r="F18" s="10" t="n"/>
-      <c r="G18" s="10" t="n"/>
-    </row>
     <row r="19">
-      <c r="A19" s="10" t="n"/>
-      <c r="B19" s="10" t="n"/>
-      <c r="C19" s="10" t="n"/>
-      <c r="D19" s="11" t="n"/>
-      <c r="E19" s="11" t="n"/>
-      <c r="F19" s="10" t="n"/>
-      <c r="G19" s="10" t="n"/>
+      <c r="A19" s="20" t="inlineStr">
+        <is>
+          <t>b018</t>
+        </is>
+      </c>
+      <c r="B19" s="20" t="inlineStr">
+        <is>
+          <t>Tender Offer</t>
+        </is>
+      </c>
+      <c r="C19" s="20" t="inlineStr">
+        <is>
+          <t>BusinessObject</t>
+        </is>
+      </c>
+      <c r="D19" s="11" t="inlineStr">
+        <is>
+          <t>Vendor response including technical proposal, pricing and references</t>
+        </is>
+      </c>
+      <c r="E19" s="11" t="inlineStr"/>
+      <c r="F19" s="20" t="inlineStr">
+        <is>
+          <t>document</t>
+        </is>
+      </c>
+      <c r="G19" s="20" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
     </row>
     <row r="20">
-      <c r="A20" s="10" t="n"/>
-      <c r="B20" s="10" t="n"/>
-      <c r="C20" s="10" t="n"/>
-      <c r="D20" s="11" t="n"/>
-      <c r="E20" s="11" t="n"/>
-      <c r="F20" s="10" t="n"/>
-      <c r="G20" s="10" t="n"/>
+      <c r="A20" s="20" t="inlineStr">
+        <is>
+          <t>b019</t>
+        </is>
+      </c>
+      <c r="B20" s="20" t="inlineStr">
+        <is>
+          <t>Award Notice</t>
+        </is>
+      </c>
+      <c r="C20" s="20" t="inlineStr">
+        <is>
+          <t>BusinessObject</t>
+        </is>
+      </c>
+      <c r="D20" s="11" t="inlineStr">
+        <is>
+          <t>Official contract award notice published on TED after standstill period</t>
+        </is>
+      </c>
+      <c r="E20" s="11" t="inlineStr"/>
+      <c r="F20" s="20" t="inlineStr">
+        <is>
+          <t>document</t>
+        </is>
+      </c>
+      <c r="G20" s="20" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
     </row>
     <row r="21">
-      <c r="A21" s="10" t="n"/>
-      <c r="B21" s="10" t="n"/>
-      <c r="C21" s="10" t="n"/>
-      <c r="D21" s="11" t="n"/>
-      <c r="E21" s="11" t="n"/>
-      <c r="F21" s="10" t="n"/>
-      <c r="G21" s="10" t="n"/>
+      <c r="A21" s="20" t="inlineStr">
+        <is>
+          <t>b020</t>
+        </is>
+      </c>
+      <c r="B21" s="20" t="inlineStr">
+        <is>
+          <t>ESB Contract</t>
+        </is>
+      </c>
+      <c r="C21" s="20" t="inlineStr">
+        <is>
+          <t>Contract</t>
+        </is>
+      </c>
+      <c r="D21" s="11" t="inlineStr">
+        <is>
+          <t>Signed contract covering licence, implementation, SLA and maintenance</t>
+        </is>
+      </c>
+      <c r="E21" s="11" t="inlineStr"/>
+      <c r="F21" s="20" t="inlineStr">
+        <is>
+          <t>document, legal</t>
+        </is>
+      </c>
+      <c r="G21" s="20" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="10" t="n"/>
@@ -1342,221 +1737,433 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="12" t="inlineStr"/>
-      <c r="B2" s="12" t="inlineStr">
-        <is>
-          <t>Order Management System</t>
-        </is>
-      </c>
-      <c r="C2" s="12" t="inlineStr">
+      <c r="A2" s="21" t="inlineStr">
+        <is>
+          <t>a001</t>
+        </is>
+      </c>
+      <c r="B2" s="21" t="inlineStr">
+        <is>
+          <t>ESB Platform</t>
+        </is>
+      </c>
+      <c r="C2" s="21" t="inlineStr">
         <is>
           <t>ApplicationComponent</t>
         </is>
       </c>
       <c r="D2" s="13" t="inlineStr">
         <is>
-          <t>Core application for order processing</t>
+          <t>Core enterprise service bus: message routing, transformation and orchestration</t>
         </is>
       </c>
       <c r="E2" s="13" t="inlineStr"/>
-      <c r="F2" s="12" t="inlineStr">
-        <is>
-          <t>core</t>
-        </is>
-      </c>
-      <c r="G2" s="12" t="inlineStr">
+      <c r="F2" s="21" t="inlineStr">
+        <is>
+          <t>core, esb</t>
+        </is>
+      </c>
+      <c r="G2" s="21" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="12" t="inlineStr"/>
-      <c r="B3" s="12" t="inlineStr">
-        <is>
-          <t>CRM System</t>
-        </is>
-      </c>
-      <c r="C3" s="12" t="inlineStr">
+      <c r="A3" s="21" t="inlineStr">
+        <is>
+          <t>a002</t>
+        </is>
+      </c>
+      <c r="B3" s="21" t="inlineStr">
+        <is>
+          <t>API Gateway</t>
+        </is>
+      </c>
+      <c r="C3" s="21" t="inlineStr">
         <is>
           <t>ApplicationComponent</t>
         </is>
       </c>
       <c r="D3" s="13" t="inlineStr">
         <is>
-          <t>Customer relationship management platform</t>
+          <t>Manages API lifecycle, security, throttling and versioning for all services</t>
         </is>
       </c>
       <c r="E3" s="13" t="inlineStr"/>
-      <c r="F3" s="12" t="inlineStr">
-        <is>
-          <t>core</t>
-        </is>
-      </c>
-      <c r="G3" s="12" t="inlineStr">
+      <c r="F3" s="21" t="inlineStr">
+        <is>
+          <t>api, security</t>
+        </is>
+      </c>
+      <c r="G3" s="21" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="12" t="inlineStr"/>
-      <c r="B4" s="12" t="inlineStr">
-        <is>
-          <t>API Gateway</t>
-        </is>
-      </c>
-      <c r="C4" s="12" t="inlineStr">
+      <c r="A4" s="21" t="inlineStr">
+        <is>
+          <t>a003</t>
+        </is>
+      </c>
+      <c r="B4" s="21" t="inlineStr">
+        <is>
+          <t>Message Broker</t>
+        </is>
+      </c>
+      <c r="C4" s="21" t="inlineStr">
         <is>
           <t>ApplicationComponent</t>
         </is>
       </c>
       <c r="D4" s="13" t="inlineStr">
         <is>
-          <t>Central API entry point for all services</t>
+          <t>Asynchronous messaging backbone (e.g. ActiveMQ, RabbitMQ)</t>
         </is>
       </c>
       <c r="E4" s="13" t="inlineStr"/>
-      <c r="F4" s="12" t="inlineStr">
-        <is>
-          <t>infrastructure</t>
-        </is>
-      </c>
-      <c r="G4" s="12" t="inlineStr">
+      <c r="F4" s="21" t="inlineStr">
+        <is>
+          <t>messaging</t>
+        </is>
+      </c>
+      <c r="G4" s="21" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="12" t="inlineStr"/>
-      <c r="B5" s="12" t="inlineStr">
-        <is>
-          <t>Order API</t>
-        </is>
-      </c>
-      <c r="C5" s="12" t="inlineStr">
-        <is>
-          <t>ApplicationInterface</t>
+      <c r="A5" s="21" t="inlineStr">
+        <is>
+          <t>a004</t>
+        </is>
+      </c>
+      <c r="B5" s="21" t="inlineStr">
+        <is>
+          <t>Service Registry</t>
+        </is>
+      </c>
+      <c r="C5" s="21" t="inlineStr">
+        <is>
+          <t>ApplicationComponent</t>
         </is>
       </c>
       <c r="D5" s="13" t="inlineStr">
         <is>
-          <t>REST API exposing order operations</t>
+          <t>Catalogue of available services, endpoints and contracts</t>
         </is>
       </c>
       <c r="E5" s="13" t="inlineStr"/>
-      <c r="F5" s="12" t="inlineStr">
-        <is>
-          <t>api</t>
-        </is>
-      </c>
-      <c r="G5" s="12" t="inlineStr">
+      <c r="F5" s="21" t="inlineStr">
+        <is>
+          <t>governance</t>
+        </is>
+      </c>
+      <c r="G5" s="21" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="12" t="inlineStr"/>
-      <c r="B6" s="12" t="inlineStr">
-        <is>
-          <t>Order Data</t>
-        </is>
-      </c>
-      <c r="C6" s="12" t="inlineStr">
+      <c r="A6" s="21" t="inlineStr">
+        <is>
+          <t>a005</t>
+        </is>
+      </c>
+      <c r="B6" s="21" t="inlineStr">
+        <is>
+          <t>Monitoring Console</t>
+        </is>
+      </c>
+      <c r="C6" s="21" t="inlineStr">
+        <is>
+          <t>ApplicationComponent</t>
+        </is>
+      </c>
+      <c r="D6" s="13" t="inlineStr">
+        <is>
+          <t>Real-time operational monitoring, alerting and SLA dashboards</t>
+        </is>
+      </c>
+      <c r="E6" s="13" t="inlineStr"/>
+      <c r="F6" s="21" t="inlineStr">
+        <is>
+          <t>operations</t>
+        </is>
+      </c>
+      <c r="G6" s="21" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="21" t="inlineStr">
+        <is>
+          <t>a006</t>
+        </is>
+      </c>
+      <c r="B7" s="21" t="inlineStr">
+        <is>
+          <t>Identity &amp; Access Mgmt</t>
+        </is>
+      </c>
+      <c r="C7" s="21" t="inlineStr">
+        <is>
+          <t>ApplicationComponent</t>
+        </is>
+      </c>
+      <c r="D7" s="13" t="inlineStr">
+        <is>
+          <t>Central IAM for service authentication and authorisation (OAuth2/SAML)</t>
+        </is>
+      </c>
+      <c r="E7" s="13" t="inlineStr"/>
+      <c r="F7" s="21" t="inlineStr">
+        <is>
+          <t>security</t>
+        </is>
+      </c>
+      <c r="G7" s="21" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="21" t="inlineStr">
+        <is>
+          <t>a007</t>
+        </is>
+      </c>
+      <c r="B8" s="21" t="inlineStr">
+        <is>
+          <t>Message Routing Service</t>
+        </is>
+      </c>
+      <c r="C8" s="21" t="inlineStr">
+        <is>
+          <t>ApplicationService</t>
+        </is>
+      </c>
+      <c r="D8" s="13" t="inlineStr">
+        <is>
+          <t>Routes messages between source and target systems based on content and rules</t>
+        </is>
+      </c>
+      <c r="E8" s="13" t="inlineStr"/>
+      <c r="F8" s="21" t="inlineStr">
+        <is>
+          <t>core, routing</t>
+        </is>
+      </c>
+      <c r="G8" s="21" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="21" t="inlineStr">
+        <is>
+          <t>a008</t>
+        </is>
+      </c>
+      <c r="B9" s="21" t="inlineStr">
+        <is>
+          <t>Data Transformation Svc</t>
+        </is>
+      </c>
+      <c r="C9" s="21" t="inlineStr">
+        <is>
+          <t>ApplicationService</t>
+        </is>
+      </c>
+      <c r="D9" s="13" t="inlineStr">
+        <is>
+          <t>Transforms data formats (XML↔JSON, canonical model mapping)</t>
+        </is>
+      </c>
+      <c r="E9" s="13" t="inlineStr"/>
+      <c r="F9" s="21" t="inlineStr">
+        <is>
+          <t>core, transformation</t>
+        </is>
+      </c>
+      <c r="G9" s="21" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="21" t="inlineStr">
+        <is>
+          <t>a009</t>
+        </is>
+      </c>
+      <c r="B10" s="21" t="inlineStr">
+        <is>
+          <t>Protocol Mediation Svc</t>
+        </is>
+      </c>
+      <c r="C10" s="21" t="inlineStr">
+        <is>
+          <t>ApplicationService</t>
+        </is>
+      </c>
+      <c r="D10" s="13" t="inlineStr">
+        <is>
+          <t>Bridges REST, SOAP, JMS, SFTP and legacy protocols</t>
+        </is>
+      </c>
+      <c r="E10" s="13" t="inlineStr"/>
+      <c r="F10" s="21" t="inlineStr">
+        <is>
+          <t>core, mediation</t>
+        </is>
+      </c>
+      <c r="G10" s="21" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="21" t="inlineStr">
+        <is>
+          <t>a010</t>
+        </is>
+      </c>
+      <c r="B11" s="21" t="inlineStr">
+        <is>
+          <t>Service Orchestration</t>
+        </is>
+      </c>
+      <c r="C11" s="21" t="inlineStr">
+        <is>
+          <t>ApplicationService</t>
+        </is>
+      </c>
+      <c r="D11" s="13" t="inlineStr">
+        <is>
+          <t>Coordinates multi-step integration flows and business processes</t>
+        </is>
+      </c>
+      <c r="E11" s="13" t="inlineStr"/>
+      <c r="F11" s="21" t="inlineStr">
+        <is>
+          <t>core, orchestration</t>
+        </is>
+      </c>
+      <c r="G11" s="21" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="21" t="inlineStr">
+        <is>
+          <t>a011</t>
+        </is>
+      </c>
+      <c r="B12" s="21" t="inlineStr">
+        <is>
+          <t>Integration Schema</t>
+        </is>
+      </c>
+      <c r="C12" s="21" t="inlineStr">
         <is>
           <t>DataObject</t>
         </is>
       </c>
-      <c r="D6" s="13" t="inlineStr">
-        <is>
-          <t>Data entity representing an order record</t>
-        </is>
-      </c>
-      <c r="E6" s="13" t="inlineStr"/>
-      <c r="F6" s="12" t="inlineStr">
-        <is>
-          <t>data</t>
-        </is>
-      </c>
-      <c r="G6" s="12" t="inlineStr">
+      <c r="D12" s="13" t="inlineStr">
+        <is>
+          <t>Canonical data model and XSD/JSON schemas for all integrated systems</t>
+        </is>
+      </c>
+      <c r="E12" s="13" t="inlineStr"/>
+      <c r="F12" s="21" t="inlineStr">
+        <is>
+          <t>data, governance</t>
+        </is>
+      </c>
+      <c r="G12" s="21" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="12" t="n"/>
-      <c r="B7" s="12" t="n"/>
-      <c r="C7" s="12" t="n"/>
-      <c r="D7" s="13" t="n"/>
-      <c r="E7" s="13" t="n"/>
-      <c r="F7" s="12" t="n"/>
-      <c r="G7" s="12" t="n"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="12" t="n"/>
-      <c r="B8" s="12" t="n"/>
-      <c r="C8" s="12" t="n"/>
-      <c r="D8" s="13" t="n"/>
-      <c r="E8" s="13" t="n"/>
-      <c r="F8" s="12" t="n"/>
-      <c r="G8" s="12" t="n"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="12" t="n"/>
-      <c r="B9" s="12" t="n"/>
-      <c r="C9" s="12" t="n"/>
-      <c r="D9" s="13" t="n"/>
-      <c r="E9" s="13" t="n"/>
-      <c r="F9" s="12" t="n"/>
-      <c r="G9" s="12" t="n"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="12" t="n"/>
-      <c r="B10" s="12" t="n"/>
-      <c r="C10" s="12" t="n"/>
-      <c r="D10" s="13" t="n"/>
-      <c r="E10" s="13" t="n"/>
-      <c r="F10" s="12" t="n"/>
-      <c r="G10" s="12" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="12" t="n"/>
-      <c r="B11" s="12" t="n"/>
-      <c r="C11" s="12" t="n"/>
-      <c r="D11" s="13" t="n"/>
-      <c r="E11" s="13" t="n"/>
-      <c r="F11" s="12" t="n"/>
-      <c r="G11" s="12" t="n"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="12" t="n"/>
-      <c r="B12" s="12" t="n"/>
-      <c r="C12" s="12" t="n"/>
-      <c r="D12" s="13" t="n"/>
-      <c r="E12" s="13" t="n"/>
-      <c r="F12" s="12" t="n"/>
-      <c r="G12" s="12" t="n"/>
-    </row>
     <row r="13">
-      <c r="A13" s="12" t="n"/>
-      <c r="B13" s="12" t="n"/>
-      <c r="C13" s="12" t="n"/>
-      <c r="D13" s="13" t="n"/>
-      <c r="E13" s="13" t="n"/>
-      <c r="F13" s="12" t="n"/>
-      <c r="G13" s="12" t="n"/>
+      <c r="A13" s="21" t="inlineStr">
+        <is>
+          <t>a012</t>
+        </is>
+      </c>
+      <c r="B13" s="21" t="inlineStr">
+        <is>
+          <t>API Specification</t>
+        </is>
+      </c>
+      <c r="C13" s="21" t="inlineStr">
+        <is>
+          <t>DataObject</t>
+        </is>
+      </c>
+      <c r="D13" s="13" t="inlineStr">
+        <is>
+          <t>OpenAPI/WSDL definitions for all exposed and consumed services</t>
+        </is>
+      </c>
+      <c r="E13" s="13" t="inlineStr"/>
+      <c r="F13" s="21" t="inlineStr">
+        <is>
+          <t>data, api</t>
+        </is>
+      </c>
+      <c r="G13" s="21" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
     </row>
     <row r="14">
-      <c r="A14" s="12" t="n"/>
-      <c r="B14" s="12" t="n"/>
-      <c r="C14" s="12" t="n"/>
-      <c r="D14" s="13" t="n"/>
-      <c r="E14" s="13" t="n"/>
-      <c r="F14" s="12" t="n"/>
-      <c r="G14" s="12" t="n"/>
+      <c r="A14" s="21" t="inlineStr">
+        <is>
+          <t>a013</t>
+        </is>
+      </c>
+      <c r="B14" s="21" t="inlineStr">
+        <is>
+          <t>SLA Definition</t>
+        </is>
+      </c>
+      <c r="C14" s="21" t="inlineStr">
+        <is>
+          <t>DataObject</t>
+        </is>
+      </c>
+      <c r="D14" s="13" t="inlineStr">
+        <is>
+          <t>Service level parameters: availability, throughput, latency, support tiers</t>
+        </is>
+      </c>
+      <c r="E14" s="13" t="inlineStr"/>
+      <c r="F14" s="21" t="inlineStr">
+        <is>
+          <t>data, governance</t>
+        </is>
+      </c>
+      <c r="G14" s="21" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="12" t="n"/>
@@ -1736,185 +2343,301 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="14" t="inlineStr"/>
-      <c r="B2" s="14" t="inlineStr">
-        <is>
-          <t>Application Server</t>
-        </is>
-      </c>
-      <c r="C2" s="14" t="inlineStr">
+      <c r="A2" s="22" t="inlineStr">
+        <is>
+          <t>t001</t>
+        </is>
+      </c>
+      <c r="B2" s="22" t="inlineStr">
+        <is>
+          <t>Integration Server</t>
+        </is>
+      </c>
+      <c r="C2" s="22" t="inlineStr">
         <is>
           <t>Node</t>
         </is>
       </c>
       <c r="D2" s="15" t="inlineStr">
         <is>
-          <t>Hosts core business applications</t>
+          <t>Primary server (on-prem or cloud VM) hosting ESB runtime</t>
         </is>
       </c>
       <c r="E2" s="15" t="inlineStr"/>
-      <c r="F2" s="14" t="inlineStr">
+      <c r="F2" s="22" t="inlineStr">
         <is>
           <t>infrastructure</t>
         </is>
       </c>
-      <c r="G2" s="14" t="inlineStr">
+      <c r="G2" s="22" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="14" t="inlineStr"/>
-      <c r="B3" s="14" t="inlineStr">
-        <is>
-          <t>Database Server</t>
-        </is>
-      </c>
-      <c r="C3" s="14" t="inlineStr">
+      <c r="A3" s="22" t="inlineStr">
+        <is>
+          <t>t002</t>
+        </is>
+      </c>
+      <c r="B3" s="22" t="inlineStr">
+        <is>
+          <t>Message Queue Server</t>
+        </is>
+      </c>
+      <c r="C3" s="22" t="inlineStr">
         <is>
           <t>Node</t>
         </is>
       </c>
       <c r="D3" s="15" t="inlineStr">
         <is>
-          <t>Relational database for transactional data</t>
+          <t>Dedicated server for async message broker and persistent queues</t>
         </is>
       </c>
       <c r="E3" s="15" t="inlineStr"/>
-      <c r="F3" s="14" t="inlineStr">
+      <c r="F3" s="22" t="inlineStr">
         <is>
           <t>infrastructure</t>
         </is>
       </c>
-      <c r="G3" s="14" t="inlineStr">
+      <c r="G3" s="22" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="14" t="inlineStr"/>
-      <c r="B4" s="14" t="inlineStr">
-        <is>
-          <t>Kubernetes Cluster</t>
-        </is>
-      </c>
-      <c r="C4" s="14" t="inlineStr">
+      <c r="A4" s="22" t="inlineStr">
+        <is>
+          <t>t003</t>
+        </is>
+      </c>
+      <c r="B4" s="22" t="inlineStr">
+        <is>
+          <t>API Gateway Server</t>
+        </is>
+      </c>
+      <c r="C4" s="22" t="inlineStr">
+        <is>
+          <t>Node</t>
+        </is>
+      </c>
+      <c r="D4" s="15" t="inlineStr">
+        <is>
+          <t>Server or load-balanced cluster hosting the API Gateway</t>
+        </is>
+      </c>
+      <c r="E4" s="15" t="inlineStr"/>
+      <c r="F4" s="22" t="inlineStr">
+        <is>
+          <t>infrastructure</t>
+        </is>
+      </c>
+      <c r="G4" s="22" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="22" t="inlineStr">
+        <is>
+          <t>t004</t>
+        </is>
+      </c>
+      <c r="B5" s="22" t="inlineStr">
+        <is>
+          <t>ESB Software Package</t>
+        </is>
+      </c>
+      <c r="C5" s="22" t="inlineStr">
         <is>
           <t>SystemSoftware</t>
         </is>
       </c>
-      <c r="D4" s="15" t="inlineStr">
-        <is>
-          <t>Container orchestration platform</t>
-        </is>
-      </c>
-      <c r="E4" s="15" t="inlineStr"/>
-      <c r="F4" s="14" t="inlineStr">
-        <is>
-          <t>infrastructure</t>
-        </is>
-      </c>
-      <c r="G4" s="14" t="inlineStr">
+      <c r="D5" s="15" t="inlineStr">
+        <is>
+          <t>Licensed ESB middleware (e.g. MuleSoft, WSO2, IBM App Connect)</t>
+        </is>
+      </c>
+      <c r="E5" s="15" t="inlineStr"/>
+      <c r="F5" s="22" t="inlineStr">
+        <is>
+          <t>software, licence</t>
+        </is>
+      </c>
+      <c r="G5" s="22" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="14" t="inlineStr"/>
-      <c r="B5" s="14" t="inlineStr">
-        <is>
-          <t>Internal Network</t>
-        </is>
-      </c>
-      <c r="C5" s="14" t="inlineStr">
+    <row r="6">
+      <c r="A6" s="22" t="inlineStr">
+        <is>
+          <t>t005</t>
+        </is>
+      </c>
+      <c r="B6" s="22" t="inlineStr">
+        <is>
+          <t>Container Platform</t>
+        </is>
+      </c>
+      <c r="C6" s="22" t="inlineStr">
+        <is>
+          <t>SystemSoftware</t>
+        </is>
+      </c>
+      <c r="D6" s="15" t="inlineStr">
+        <is>
+          <t>Docker/Kubernetes for containerised ESB deployment and scaling</t>
+        </is>
+      </c>
+      <c r="E6" s="15" t="inlineStr"/>
+      <c r="F6" s="22" t="inlineStr">
+        <is>
+          <t>software, infra</t>
+        </is>
+      </c>
+      <c r="G6" s="22" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="22" t="inlineStr">
+        <is>
+          <t>t006</t>
+        </is>
+      </c>
+      <c r="B7" s="22" t="inlineStr">
+        <is>
+          <t>Operating System</t>
+        </is>
+      </c>
+      <c r="C7" s="22" t="inlineStr">
+        <is>
+          <t>SystemSoftware</t>
+        </is>
+      </c>
+      <c r="D7" s="15" t="inlineStr">
+        <is>
+          <t>RHEL or Ubuntu LTS; hardened per municipal security baseline</t>
+        </is>
+      </c>
+      <c r="E7" s="15" t="inlineStr"/>
+      <c r="F7" s="22" t="inlineStr">
+        <is>
+          <t>software</t>
+        </is>
+      </c>
+      <c r="G7" s="22" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="22" t="inlineStr">
+        <is>
+          <t>t007</t>
+        </is>
+      </c>
+      <c r="B8" s="22" t="inlineStr">
+        <is>
+          <t>Municipal Network</t>
+        </is>
+      </c>
+      <c r="C8" s="22" t="inlineStr">
         <is>
           <t>CommunicationNetwork</t>
         </is>
       </c>
-      <c r="D5" s="15" t="inlineStr">
-        <is>
-          <t>Internal corporate network</t>
-        </is>
-      </c>
-      <c r="E5" s="15" t="inlineStr"/>
-      <c r="F5" s="14" t="inlineStr">
+      <c r="D8" s="15" t="inlineStr">
+        <is>
+          <t>Internal municipal LAN/WAN connecting all back-office systems</t>
+        </is>
+      </c>
+      <c r="E8" s="15" t="inlineStr"/>
+      <c r="F8" s="22" t="inlineStr">
         <is>
           <t>network</t>
         </is>
       </c>
-      <c r="G5" s="14" t="inlineStr">
+      <c r="G8" s="22" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="14" t="inlineStr"/>
-      <c r="B6" s="14" t="inlineStr">
-        <is>
-          <t>PostgreSQL</t>
-        </is>
-      </c>
-      <c r="C6" s="14" t="inlineStr">
-        <is>
-          <t>SystemSoftware</t>
-        </is>
-      </c>
-      <c r="D6" s="15" t="inlineStr">
-        <is>
-          <t>Primary relational database engine</t>
-        </is>
-      </c>
-      <c r="E6" s="15" t="inlineStr"/>
-      <c r="F6" s="14" t="inlineStr">
-        <is>
-          <t>database</t>
-        </is>
-      </c>
-      <c r="G6" s="14" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="22" t="inlineStr">
+        <is>
+          <t>t008</t>
+        </is>
+      </c>
+      <c r="B9" s="22" t="inlineStr">
+        <is>
+          <t>DMZ</t>
+        </is>
+      </c>
+      <c r="C9" s="22" t="inlineStr">
+        <is>
+          <t>CommunicationNetwork</t>
+        </is>
+      </c>
+      <c r="D9" s="15" t="inlineStr">
+        <is>
+          <t>Demilitarised zone for controlled external partner access to ESB APIs</t>
+        </is>
+      </c>
+      <c r="E9" s="15" t="inlineStr"/>
+      <c r="F9" s="22" t="inlineStr">
+        <is>
+          <t>network, security</t>
+        </is>
+      </c>
+      <c r="G9" s="22" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="14" t="n"/>
-      <c r="B7" s="14" t="n"/>
-      <c r="C7" s="14" t="n"/>
-      <c r="D7" s="15" t="n"/>
-      <c r="E7" s="15" t="n"/>
-      <c r="F7" s="14" t="n"/>
-      <c r="G7" s="14" t="n"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="14" t="n"/>
-      <c r="B8" s="14" t="n"/>
-      <c r="C8" s="14" t="n"/>
-      <c r="D8" s="15" t="n"/>
-      <c r="E8" s="15" t="n"/>
-      <c r="F8" s="14" t="n"/>
-      <c r="G8" s="14" t="n"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="14" t="n"/>
-      <c r="B9" s="14" t="n"/>
-      <c r="C9" s="14" t="n"/>
-      <c r="D9" s="15" t="n"/>
-      <c r="E9" s="15" t="n"/>
-      <c r="F9" s="14" t="n"/>
-      <c r="G9" s="14" t="n"/>
-    </row>
     <row r="10">
-      <c r="A10" s="14" t="n"/>
-      <c r="B10" s="14" t="n"/>
-      <c r="C10" s="14" t="n"/>
-      <c r="D10" s="15" t="n"/>
-      <c r="E10" s="15" t="n"/>
-      <c r="F10" s="14" t="n"/>
-      <c r="G10" s="14" t="n"/>
+      <c r="A10" s="22" t="inlineStr">
+        <is>
+          <t>t009</t>
+        </is>
+      </c>
+      <c r="B10" s="22" t="inlineStr">
+        <is>
+          <t>Deployment Package</t>
+        </is>
+      </c>
+      <c r="C10" s="22" t="inlineStr">
+        <is>
+          <t>Artifact</t>
+        </is>
+      </c>
+      <c r="D10" s="15" t="inlineStr">
+        <is>
+          <t>ESB installation scripts, Helm charts and configuration artefacts</t>
+        </is>
+      </c>
+      <c r="E10" s="15" t="inlineStr"/>
+      <c r="F10" s="22" t="inlineStr">
+        <is>
+          <t>devops</t>
+        </is>
+      </c>
+      <c r="G10" s="22" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="14" t="n"/>
@@ -2080,7 +2803,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I26"/>
+  <dimension ref="A1:I52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -2142,379 +2865,1609 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="16" t="inlineStr"/>
-      <c r="B2" s="16" t="inlineStr">
-        <is>
-          <t>&lt;Business Actor ID&gt;</t>
-        </is>
-      </c>
-      <c r="C2" s="16" t="inlineStr">
-        <is>
-          <t>Customer</t>
+      <c r="A2" s="23" t="inlineStr"/>
+      <c r="B2" s="23" t="inlineStr">
+        <is>
+          <t>b001</t>
+        </is>
+      </c>
+      <c r="C2" s="23" t="inlineStr">
+        <is>
+          <t>Municipality</t>
         </is>
       </c>
       <c r="D2" s="17" t="inlineStr">
         <is>
-          <t>&lt;Business Role ID&gt;</t>
+          <t>b004</t>
         </is>
       </c>
       <c r="E2" s="17" t="inlineStr">
         <is>
-          <t>Account Manager</t>
-        </is>
-      </c>
-      <c r="F2" s="16" t="inlineStr">
+          <t>Contracting Officer</t>
+        </is>
+      </c>
+      <c r="F2" s="23" t="inlineStr">
+        <is>
+          <t>AssignmentRelationship</t>
+        </is>
+      </c>
+      <c r="G2" s="23" t="inlineStr"/>
+      <c r="H2" s="23" t="inlineStr"/>
+      <c r="I2" s="23" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="23" t="inlineStr"/>
+      <c r="B3" s="23" t="inlineStr">
+        <is>
+          <t>b001</t>
+        </is>
+      </c>
+      <c r="C3" s="23" t="inlineStr">
+        <is>
+          <t>Municipality</t>
+        </is>
+      </c>
+      <c r="D3" s="17" t="inlineStr">
+        <is>
+          <t>b005</t>
+        </is>
+      </c>
+      <c r="E3" s="17" t="inlineStr">
+        <is>
+          <t>IT Architect</t>
+        </is>
+      </c>
+      <c r="F3" s="23" t="inlineStr">
+        <is>
+          <t>AssignmentRelationship</t>
+        </is>
+      </c>
+      <c r="G3" s="23" t="inlineStr"/>
+      <c r="H3" s="23" t="inlineStr"/>
+      <c r="I3" s="23" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="23" t="inlineStr"/>
+      <c r="B4" s="23" t="inlineStr">
+        <is>
+          <t>b001</t>
+        </is>
+      </c>
+      <c r="C4" s="23" t="inlineStr">
+        <is>
+          <t>Municipality</t>
+        </is>
+      </c>
+      <c r="D4" s="17" t="inlineStr">
+        <is>
+          <t>b006</t>
+        </is>
+      </c>
+      <c r="E4" s="17" t="inlineStr">
+        <is>
+          <t>Legal Advisor</t>
+        </is>
+      </c>
+      <c r="F4" s="23" t="inlineStr">
+        <is>
+          <t>AssignmentRelationship</t>
+        </is>
+      </c>
+      <c r="G4" s="23" t="inlineStr"/>
+      <c r="H4" s="23" t="inlineStr"/>
+      <c r="I4" s="23" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="23" t="inlineStr"/>
+      <c r="B5" s="23" t="inlineStr">
+        <is>
+          <t>b003</t>
+        </is>
+      </c>
+      <c r="C5" s="23" t="inlineStr">
+        <is>
+          <t>Evaluation Committee</t>
+        </is>
+      </c>
+      <c r="D5" s="17" t="inlineStr">
+        <is>
+          <t>b004</t>
+        </is>
+      </c>
+      <c r="E5" s="17" t="inlineStr">
+        <is>
+          <t>Contracting Officer</t>
+        </is>
+      </c>
+      <c r="F5" s="23" t="inlineStr">
+        <is>
+          <t>AggregationRelationship</t>
+        </is>
+      </c>
+      <c r="G5" s="23" t="inlineStr"/>
+      <c r="H5" s="23" t="inlineStr"/>
+      <c r="I5" s="23" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="23" t="inlineStr"/>
+      <c r="B6" s="23" t="inlineStr">
+        <is>
+          <t>b003</t>
+        </is>
+      </c>
+      <c r="C6" s="23" t="inlineStr">
+        <is>
+          <t>Evaluation Committee</t>
+        </is>
+      </c>
+      <c r="D6" s="17" t="inlineStr">
+        <is>
+          <t>b005</t>
+        </is>
+      </c>
+      <c r="E6" s="17" t="inlineStr">
+        <is>
+          <t>IT Architect</t>
+        </is>
+      </c>
+      <c r="F6" s="23" t="inlineStr">
+        <is>
+          <t>AggregationRelationship</t>
+        </is>
+      </c>
+      <c r="G6" s="23" t="inlineStr"/>
+      <c r="H6" s="23" t="inlineStr"/>
+      <c r="I6" s="23" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="23" t="inlineStr"/>
+      <c r="B7" s="23" t="inlineStr">
+        <is>
+          <t>b007</t>
+        </is>
+      </c>
+      <c r="C7" s="23" t="inlineStr">
+        <is>
+          <t>Needs Assessment</t>
+        </is>
+      </c>
+      <c r="D7" s="17" t="inlineStr">
+        <is>
+          <t>b008</t>
+        </is>
+      </c>
+      <c r="E7" s="17" t="inlineStr">
+        <is>
+          <t>Market Consultation</t>
+        </is>
+      </c>
+      <c r="F7" s="23" t="inlineStr">
+        <is>
+          <t>TriggeringRelationship</t>
+        </is>
+      </c>
+      <c r="G7" s="23" t="inlineStr"/>
+      <c r="H7" s="23" t="inlineStr"/>
+      <c r="I7" s="23" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="23" t="inlineStr"/>
+      <c r="B8" s="23" t="inlineStr">
+        <is>
+          <t>b008</t>
+        </is>
+      </c>
+      <c r="C8" s="23" t="inlineStr">
+        <is>
+          <t>Market Consultation</t>
+        </is>
+      </c>
+      <c r="D8" s="17" t="inlineStr">
+        <is>
+          <t>b009</t>
+        </is>
+      </c>
+      <c r="E8" s="17" t="inlineStr">
+        <is>
+          <t>Tender Preparation</t>
+        </is>
+      </c>
+      <c r="F8" s="23" t="inlineStr">
+        <is>
+          <t>TriggeringRelationship</t>
+        </is>
+      </c>
+      <c r="G8" s="23" t="inlineStr"/>
+      <c r="H8" s="23" t="inlineStr"/>
+      <c r="I8" s="23" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="23" t="inlineStr"/>
+      <c r="B9" s="23" t="inlineStr">
+        <is>
+          <t>b009</t>
+        </is>
+      </c>
+      <c r="C9" s="23" t="inlineStr">
+        <is>
+          <t>Tender Preparation</t>
+        </is>
+      </c>
+      <c r="D9" s="17" t="inlineStr">
+        <is>
+          <t>b010</t>
+        </is>
+      </c>
+      <c r="E9" s="17" t="inlineStr">
+        <is>
+          <t>Tender Publication</t>
+        </is>
+      </c>
+      <c r="F9" s="23" t="inlineStr">
+        <is>
+          <t>TriggeringRelationship</t>
+        </is>
+      </c>
+      <c r="G9" s="23" t="inlineStr"/>
+      <c r="H9" s="23" t="inlineStr"/>
+      <c r="I9" s="23" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="23" t="inlineStr"/>
+      <c r="B10" s="23" t="inlineStr">
+        <is>
+          <t>b010</t>
+        </is>
+      </c>
+      <c r="C10" s="23" t="inlineStr">
+        <is>
+          <t>Tender Publication</t>
+        </is>
+      </c>
+      <c r="D10" s="17" t="inlineStr">
+        <is>
+          <t>b011</t>
+        </is>
+      </c>
+      <c r="E10" s="17" t="inlineStr">
+        <is>
+          <t>Tender Reception</t>
+        </is>
+      </c>
+      <c r="F10" s="23" t="inlineStr">
+        <is>
+          <t>TriggeringRelationship</t>
+        </is>
+      </c>
+      <c r="G10" s="23" t="inlineStr"/>
+      <c r="H10" s="23" t="inlineStr"/>
+      <c r="I10" s="23" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="23" t="inlineStr"/>
+      <c r="B11" s="23" t="inlineStr">
+        <is>
+          <t>b011</t>
+        </is>
+      </c>
+      <c r="C11" s="23" t="inlineStr">
+        <is>
+          <t>Tender Reception</t>
+        </is>
+      </c>
+      <c r="D11" s="17" t="inlineStr">
+        <is>
+          <t>b012</t>
+        </is>
+      </c>
+      <c r="E11" s="17" t="inlineStr">
+        <is>
+          <t>Tender Evaluation</t>
+        </is>
+      </c>
+      <c r="F11" s="23" t="inlineStr">
+        <is>
+          <t>TriggeringRelationship</t>
+        </is>
+      </c>
+      <c r="G11" s="23" t="inlineStr"/>
+      <c r="H11" s="23" t="inlineStr"/>
+      <c r="I11" s="23" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="23" t="inlineStr"/>
+      <c r="B12" s="23" t="inlineStr">
+        <is>
+          <t>b012</t>
+        </is>
+      </c>
+      <c r="C12" s="23" t="inlineStr">
+        <is>
+          <t>Tender Evaluation</t>
+        </is>
+      </c>
+      <c r="D12" s="17" t="inlineStr">
+        <is>
+          <t>b013</t>
+        </is>
+      </c>
+      <c r="E12" s="17" t="inlineStr">
+        <is>
+          <t>Contract Award</t>
+        </is>
+      </c>
+      <c r="F12" s="23" t="inlineStr">
+        <is>
+          <t>TriggeringRelationship</t>
+        </is>
+      </c>
+      <c r="G12" s="23" t="inlineStr"/>
+      <c r="H12" s="23" t="inlineStr"/>
+      <c r="I12" s="23" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="23" t="inlineStr"/>
+      <c r="B13" s="23" t="inlineStr">
+        <is>
+          <t>b013</t>
+        </is>
+      </c>
+      <c r="C13" s="23" t="inlineStr">
+        <is>
+          <t>Contract Award</t>
+        </is>
+      </c>
+      <c r="D13" s="17" t="inlineStr">
+        <is>
+          <t>b014</t>
+        </is>
+      </c>
+      <c r="E13" s="17" t="inlineStr">
+        <is>
+          <t>ESB Implementation</t>
+        </is>
+      </c>
+      <c r="F13" s="23" t="inlineStr">
+        <is>
+          <t>TriggeringRelationship</t>
+        </is>
+      </c>
+      <c r="G13" s="23" t="inlineStr"/>
+      <c r="H13" s="23" t="inlineStr"/>
+      <c r="I13" s="23" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="23" t="inlineStr"/>
+      <c r="B14" s="23" t="inlineStr">
+        <is>
+          <t>b014</t>
+        </is>
+      </c>
+      <c r="C14" s="23" t="inlineStr">
+        <is>
+          <t>ESB Implementation</t>
+        </is>
+      </c>
+      <c r="D14" s="17" t="inlineStr">
+        <is>
+          <t>b015</t>
+        </is>
+      </c>
+      <c r="E14" s="17" t="inlineStr">
+        <is>
+          <t>Acceptance Testing</t>
+        </is>
+      </c>
+      <c r="F14" s="23" t="inlineStr">
+        <is>
+          <t>TriggeringRelationship</t>
+        </is>
+      </c>
+      <c r="G14" s="23" t="inlineStr"/>
+      <c r="H14" s="23" t="inlineStr"/>
+      <c r="I14" s="23" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="23" t="inlineStr"/>
+      <c r="B15" s="23" t="inlineStr">
+        <is>
+          <t>b004</t>
+        </is>
+      </c>
+      <c r="C15" s="23" t="inlineStr">
+        <is>
+          <t>Contracting Officer</t>
+        </is>
+      </c>
+      <c r="D15" s="17" t="inlineStr">
+        <is>
+          <t>b010</t>
+        </is>
+      </c>
+      <c r="E15" s="17" t="inlineStr">
+        <is>
+          <t>Tender Publication</t>
+        </is>
+      </c>
+      <c r="F15" s="23" t="inlineStr">
+        <is>
+          <t>AssignmentRelationship</t>
+        </is>
+      </c>
+      <c r="G15" s="23" t="inlineStr"/>
+      <c r="H15" s="23" t="inlineStr"/>
+      <c r="I15" s="23" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="23" t="inlineStr"/>
+      <c r="B16" s="23" t="inlineStr">
+        <is>
+          <t>b004</t>
+        </is>
+      </c>
+      <c r="C16" s="23" t="inlineStr">
+        <is>
+          <t>Contracting Officer</t>
+        </is>
+      </c>
+      <c r="D16" s="17" t="inlineStr">
+        <is>
+          <t>b013</t>
+        </is>
+      </c>
+      <c r="E16" s="17" t="inlineStr">
+        <is>
+          <t>Contract Award</t>
+        </is>
+      </c>
+      <c r="F16" s="23" t="inlineStr">
+        <is>
+          <t>AssignmentRelationship</t>
+        </is>
+      </c>
+      <c r="G16" s="23" t="inlineStr"/>
+      <c r="H16" s="23" t="inlineStr"/>
+      <c r="I16" s="23" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="23" t="inlineStr"/>
+      <c r="B17" s="23" t="inlineStr">
+        <is>
+          <t>b005</t>
+        </is>
+      </c>
+      <c r="C17" s="23" t="inlineStr">
+        <is>
+          <t>IT Architect</t>
+        </is>
+      </c>
+      <c r="D17" s="17" t="inlineStr">
+        <is>
+          <t>b007</t>
+        </is>
+      </c>
+      <c r="E17" s="17" t="inlineStr">
+        <is>
+          <t>Needs Assessment</t>
+        </is>
+      </c>
+      <c r="F17" s="23" t="inlineStr">
+        <is>
+          <t>AssignmentRelationship</t>
+        </is>
+      </c>
+      <c r="G17" s="23" t="inlineStr"/>
+      <c r="H17" s="23" t="inlineStr"/>
+      <c r="I17" s="23" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="23" t="inlineStr"/>
+      <c r="B18" s="23" t="inlineStr">
+        <is>
+          <t>b005</t>
+        </is>
+      </c>
+      <c r="C18" s="23" t="inlineStr">
+        <is>
+          <t>IT Architect</t>
+        </is>
+      </c>
+      <c r="D18" s="17" t="inlineStr">
+        <is>
+          <t>b009</t>
+        </is>
+      </c>
+      <c r="E18" s="17" t="inlineStr">
+        <is>
+          <t>Tender Preparation</t>
+        </is>
+      </c>
+      <c r="F18" s="23" t="inlineStr">
+        <is>
+          <t>AssignmentRelationship</t>
+        </is>
+      </c>
+      <c r="G18" s="23" t="inlineStr"/>
+      <c r="H18" s="23" t="inlineStr"/>
+      <c r="I18" s="23" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="23" t="inlineStr"/>
+      <c r="B19" s="23" t="inlineStr">
+        <is>
+          <t>b006</t>
+        </is>
+      </c>
+      <c r="C19" s="23" t="inlineStr">
+        <is>
+          <t>Legal Advisor</t>
+        </is>
+      </c>
+      <c r="D19" s="17" t="inlineStr">
+        <is>
+          <t>b009</t>
+        </is>
+      </c>
+      <c r="E19" s="17" t="inlineStr">
+        <is>
+          <t>Tender Preparation</t>
+        </is>
+      </c>
+      <c r="F19" s="23" t="inlineStr">
+        <is>
+          <t>AssignmentRelationship</t>
+        </is>
+      </c>
+      <c r="G19" s="23" t="inlineStr"/>
+      <c r="H19" s="23" t="inlineStr"/>
+      <c r="I19" s="23" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="23" t="inlineStr"/>
+      <c r="B20" s="23" t="inlineStr">
+        <is>
+          <t>b006</t>
+        </is>
+      </c>
+      <c r="C20" s="23" t="inlineStr">
+        <is>
+          <t>Legal Advisor</t>
+        </is>
+      </c>
+      <c r="D20" s="17" t="inlineStr">
+        <is>
+          <t>b012</t>
+        </is>
+      </c>
+      <c r="E20" s="17" t="inlineStr">
+        <is>
+          <t>Tender Evaluation</t>
+        </is>
+      </c>
+      <c r="F20" s="23" t="inlineStr">
+        <is>
+          <t>AssignmentRelationship</t>
+        </is>
+      </c>
+      <c r="G20" s="23" t="inlineStr"/>
+      <c r="H20" s="23" t="inlineStr"/>
+      <c r="I20" s="23" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="23" t="inlineStr"/>
+      <c r="B21" s="23" t="inlineStr">
+        <is>
+          <t>b009</t>
+        </is>
+      </c>
+      <c r="C21" s="23" t="inlineStr">
+        <is>
+          <t>Tender Preparation</t>
+        </is>
+      </c>
+      <c r="D21" s="17" t="inlineStr">
+        <is>
+          <t>b017</t>
+        </is>
+      </c>
+      <c r="E21" s="17" t="inlineStr">
+        <is>
+          <t>Technical Spec</t>
+        </is>
+      </c>
+      <c r="F21" s="23" t="inlineStr">
+        <is>
+          <t>AccessRelationship</t>
+        </is>
+      </c>
+      <c r="G21" s="23" t="inlineStr">
+        <is>
+          <t>write</t>
+        </is>
+      </c>
+      <c r="H21" s="23" t="inlineStr"/>
+      <c r="I21" s="23" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="23" t="inlineStr"/>
+      <c r="B22" s="23" t="inlineStr">
+        <is>
+          <t>b012</t>
+        </is>
+      </c>
+      <c r="C22" s="23" t="inlineStr">
+        <is>
+          <t>Tender Evaluation</t>
+        </is>
+      </c>
+      <c r="D22" s="17" t="inlineStr">
+        <is>
+          <t>b017</t>
+        </is>
+      </c>
+      <c r="E22" s="17" t="inlineStr">
+        <is>
+          <t>Technical Spec</t>
+        </is>
+      </c>
+      <c r="F22" s="23" t="inlineStr">
+        <is>
+          <t>AccessRelationship</t>
+        </is>
+      </c>
+      <c r="G22" s="23" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="H22" s="23" t="inlineStr"/>
+      <c r="I22" s="23" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="23" t="inlineStr"/>
+      <c r="B23" s="23" t="inlineStr">
+        <is>
+          <t>b002</t>
+        </is>
+      </c>
+      <c r="C23" s="23" t="inlineStr">
+        <is>
+          <t>ESB Vendor</t>
+        </is>
+      </c>
+      <c r="D23" s="17" t="inlineStr">
+        <is>
+          <t>b018</t>
+        </is>
+      </c>
+      <c r="E23" s="17" t="inlineStr">
+        <is>
+          <t>Tender Offer</t>
+        </is>
+      </c>
+      <c r="F23" s="23" t="inlineStr">
+        <is>
+          <t>AccessRelationship</t>
+        </is>
+      </c>
+      <c r="G23" s="23" t="inlineStr">
+        <is>
+          <t>write</t>
+        </is>
+      </c>
+      <c r="H23" s="23" t="inlineStr"/>
+      <c r="I23" s="23" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="23" t="inlineStr"/>
+      <c r="B24" s="23" t="inlineStr">
+        <is>
+          <t>b012</t>
+        </is>
+      </c>
+      <c r="C24" s="23" t="inlineStr">
+        <is>
+          <t>Tender Evaluation</t>
+        </is>
+      </c>
+      <c r="D24" s="17" t="inlineStr">
+        <is>
+          <t>b018</t>
+        </is>
+      </c>
+      <c r="E24" s="17" t="inlineStr">
+        <is>
+          <t>Tender Offer</t>
+        </is>
+      </c>
+      <c r="F24" s="23" t="inlineStr">
+        <is>
+          <t>AccessRelationship</t>
+        </is>
+      </c>
+      <c r="G24" s="23" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="H24" s="23" t="inlineStr"/>
+      <c r="I24" s="23" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="23" t="inlineStr"/>
+      <c r="B25" s="23" t="inlineStr">
+        <is>
+          <t>b013</t>
+        </is>
+      </c>
+      <c r="C25" s="23" t="inlineStr">
+        <is>
+          <t>Contract Award</t>
+        </is>
+      </c>
+      <c r="D25" s="17" t="inlineStr">
+        <is>
+          <t>b019</t>
+        </is>
+      </c>
+      <c r="E25" s="17" t="inlineStr">
+        <is>
+          <t>Award Notice</t>
+        </is>
+      </c>
+      <c r="F25" s="23" t="inlineStr">
+        <is>
+          <t>AccessRelationship</t>
+        </is>
+      </c>
+      <c r="G25" s="23" t="inlineStr">
+        <is>
+          <t>write</t>
+        </is>
+      </c>
+      <c r="H25" s="23" t="inlineStr"/>
+      <c r="I25" s="23" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="23" t="inlineStr"/>
+      <c r="B26" s="23" t="inlineStr">
+        <is>
+          <t>b013</t>
+        </is>
+      </c>
+      <c r="C26" s="23" t="inlineStr">
+        <is>
+          <t>Contract Award</t>
+        </is>
+      </c>
+      <c r="D26" s="17" t="inlineStr">
+        <is>
+          <t>b020</t>
+        </is>
+      </c>
+      <c r="E26" s="17" t="inlineStr">
+        <is>
+          <t>ESB Contract</t>
+        </is>
+      </c>
+      <c r="F26" s="23" t="inlineStr">
+        <is>
+          <t>AccessRelationship</t>
+        </is>
+      </c>
+      <c r="G26" s="23" t="inlineStr">
+        <is>
+          <t>write</t>
+        </is>
+      </c>
+      <c r="H26" s="23" t="inlineStr"/>
+      <c r="I26" s="23" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="23" t="inlineStr"/>
+      <c r="B27" s="23" t="inlineStr">
+        <is>
+          <t>b014</t>
+        </is>
+      </c>
+      <c r="C27" s="23" t="inlineStr">
+        <is>
+          <t>ESB Implementation</t>
+        </is>
+      </c>
+      <c r="D27" s="17" t="inlineStr">
+        <is>
+          <t>a001</t>
+        </is>
+      </c>
+      <c r="E27" s="17" t="inlineStr">
+        <is>
+          <t>ESB Platform</t>
+        </is>
+      </c>
+      <c r="F27" s="23" t="inlineStr">
+        <is>
+          <t>RealizationRelationship</t>
+        </is>
+      </c>
+      <c r="G27" s="23" t="inlineStr"/>
+      <c r="H27" s="23" t="inlineStr"/>
+      <c r="I27" s="23" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="23" t="inlineStr"/>
+      <c r="B28" s="23" t="inlineStr">
+        <is>
+          <t>b016</t>
+        </is>
+      </c>
+      <c r="C28" s="23" t="inlineStr">
+        <is>
+          <t>Procurement Service</t>
+        </is>
+      </c>
+      <c r="D28" s="17" t="inlineStr">
+        <is>
+          <t>b001</t>
+        </is>
+      </c>
+      <c r="E28" s="17" t="inlineStr">
+        <is>
+          <t>Municipality</t>
+        </is>
+      </c>
+      <c r="F28" s="23" t="inlineStr">
+        <is>
+          <t>ServingRelationship</t>
+        </is>
+      </c>
+      <c r="G28" s="23" t="inlineStr"/>
+      <c r="H28" s="23" t="inlineStr"/>
+      <c r="I28" s="23" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="23" t="inlineStr"/>
+      <c r="B29" s="23" t="inlineStr">
+        <is>
+          <t>a001</t>
+        </is>
+      </c>
+      <c r="C29" s="23" t="inlineStr">
+        <is>
+          <t>ESB Platform</t>
+        </is>
+      </c>
+      <c r="D29" s="17" t="inlineStr">
+        <is>
+          <t>a007</t>
+        </is>
+      </c>
+      <c r="E29" s="17" t="inlineStr">
+        <is>
+          <t>Message Routing Svc</t>
+        </is>
+      </c>
+      <c r="F29" s="23" t="inlineStr">
+        <is>
+          <t>RealizationRelationship</t>
+        </is>
+      </c>
+      <c r="G29" s="23" t="inlineStr"/>
+      <c r="H29" s="23" t="inlineStr"/>
+      <c r="I29" s="23" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="23" t="inlineStr"/>
+      <c r="B30" s="23" t="inlineStr">
+        <is>
+          <t>a001</t>
+        </is>
+      </c>
+      <c r="C30" s="23" t="inlineStr">
+        <is>
+          <t>ESB Platform</t>
+        </is>
+      </c>
+      <c r="D30" s="17" t="inlineStr">
+        <is>
+          <t>a008</t>
+        </is>
+      </c>
+      <c r="E30" s="17" t="inlineStr">
+        <is>
+          <t>Data Transformation</t>
+        </is>
+      </c>
+      <c r="F30" s="23" t="inlineStr">
+        <is>
+          <t>RealizationRelationship</t>
+        </is>
+      </c>
+      <c r="G30" s="23" t="inlineStr"/>
+      <c r="H30" s="23" t="inlineStr"/>
+      <c r="I30" s="23" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="23" t="inlineStr"/>
+      <c r="B31" s="23" t="inlineStr">
+        <is>
+          <t>a001</t>
+        </is>
+      </c>
+      <c r="C31" s="23" t="inlineStr">
+        <is>
+          <t>ESB Platform</t>
+        </is>
+      </c>
+      <c r="D31" s="17" t="inlineStr">
+        <is>
+          <t>a009</t>
+        </is>
+      </c>
+      <c r="E31" s="17" t="inlineStr">
+        <is>
+          <t>Protocol Mediation</t>
+        </is>
+      </c>
+      <c r="F31" s="23" t="inlineStr">
+        <is>
+          <t>RealizationRelationship</t>
+        </is>
+      </c>
+      <c r="G31" s="23" t="inlineStr"/>
+      <c r="H31" s="23" t="inlineStr"/>
+      <c r="I31" s="23" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="23" t="inlineStr"/>
+      <c r="B32" s="23" t="inlineStr">
+        <is>
+          <t>a001</t>
+        </is>
+      </c>
+      <c r="C32" s="23" t="inlineStr">
+        <is>
+          <t>ESB Platform</t>
+        </is>
+      </c>
+      <c r="D32" s="17" t="inlineStr">
+        <is>
+          <t>a010</t>
+        </is>
+      </c>
+      <c r="E32" s="17" t="inlineStr">
+        <is>
+          <t>Service Orchestration</t>
+        </is>
+      </c>
+      <c r="F32" s="23" t="inlineStr">
+        <is>
+          <t>RealizationRelationship</t>
+        </is>
+      </c>
+      <c r="G32" s="23" t="inlineStr"/>
+      <c r="H32" s="23" t="inlineStr"/>
+      <c r="I32" s="23" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="23" t="inlineStr"/>
+      <c r="B33" s="23" t="inlineStr">
+        <is>
+          <t>a002</t>
+        </is>
+      </c>
+      <c r="C33" s="23" t="inlineStr">
+        <is>
+          <t>API Gateway</t>
+        </is>
+      </c>
+      <c r="D33" s="17" t="inlineStr">
+        <is>
+          <t>a001</t>
+        </is>
+      </c>
+      <c r="E33" s="17" t="inlineStr">
+        <is>
+          <t>ESB Platform</t>
+        </is>
+      </c>
+      <c r="F33" s="23" t="inlineStr">
+        <is>
+          <t>ServingRelationship</t>
+        </is>
+      </c>
+      <c r="G33" s="23" t="inlineStr"/>
+      <c r="H33" s="23" t="inlineStr"/>
+      <c r="I33" s="23" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="23" t="inlineStr"/>
+      <c r="B34" s="23" t="inlineStr">
+        <is>
+          <t>a003</t>
+        </is>
+      </c>
+      <c r="C34" s="23" t="inlineStr">
+        <is>
+          <t>Message Broker</t>
+        </is>
+      </c>
+      <c r="D34" s="17" t="inlineStr">
+        <is>
+          <t>a001</t>
+        </is>
+      </c>
+      <c r="E34" s="17" t="inlineStr">
+        <is>
+          <t>ESB Platform</t>
+        </is>
+      </c>
+      <c r="F34" s="23" t="inlineStr">
+        <is>
+          <t>ServingRelationship</t>
+        </is>
+      </c>
+      <c r="G34" s="23" t="inlineStr"/>
+      <c r="H34" s="23" t="inlineStr"/>
+      <c r="I34" s="23" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="23" t="inlineStr"/>
+      <c r="B35" s="23" t="inlineStr">
+        <is>
+          <t>a004</t>
+        </is>
+      </c>
+      <c r="C35" s="23" t="inlineStr">
+        <is>
+          <t>Service Registry</t>
+        </is>
+      </c>
+      <c r="D35" s="17" t="inlineStr">
+        <is>
+          <t>a001</t>
+        </is>
+      </c>
+      <c r="E35" s="17" t="inlineStr">
+        <is>
+          <t>ESB Platform</t>
+        </is>
+      </c>
+      <c r="F35" s="23" t="inlineStr">
+        <is>
+          <t>ServingRelationship</t>
+        </is>
+      </c>
+      <c r="G35" s="23" t="inlineStr"/>
+      <c r="H35" s="23" t="inlineStr"/>
+      <c r="I35" s="23" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="23" t="inlineStr"/>
+      <c r="B36" s="23" t="inlineStr">
+        <is>
+          <t>a006</t>
+        </is>
+      </c>
+      <c r="C36" s="23" t="inlineStr">
+        <is>
+          <t>IAM</t>
+        </is>
+      </c>
+      <c r="D36" s="17" t="inlineStr">
+        <is>
+          <t>a001</t>
+        </is>
+      </c>
+      <c r="E36" s="17" t="inlineStr">
+        <is>
+          <t>ESB Platform</t>
+        </is>
+      </c>
+      <c r="F36" s="23" t="inlineStr">
+        <is>
+          <t>ServingRelationship</t>
+        </is>
+      </c>
+      <c r="G36" s="23" t="inlineStr"/>
+      <c r="H36" s="23" t="inlineStr"/>
+      <c r="I36" s="23" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="23" t="inlineStr"/>
+      <c r="B37" s="23" t="inlineStr">
+        <is>
+          <t>a006</t>
+        </is>
+      </c>
+      <c r="C37" s="23" t="inlineStr">
+        <is>
+          <t>IAM</t>
+        </is>
+      </c>
+      <c r="D37" s="17" t="inlineStr">
+        <is>
+          <t>a002</t>
+        </is>
+      </c>
+      <c r="E37" s="17" t="inlineStr">
+        <is>
+          <t>API Gateway</t>
+        </is>
+      </c>
+      <c r="F37" s="23" t="inlineStr">
+        <is>
+          <t>ServingRelationship</t>
+        </is>
+      </c>
+      <c r="G37" s="23" t="inlineStr"/>
+      <c r="H37" s="23" t="inlineStr"/>
+      <c r="I37" s="23" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="23" t="inlineStr"/>
+      <c r="B38" s="23" t="inlineStr">
+        <is>
+          <t>a005</t>
+        </is>
+      </c>
+      <c r="C38" s="23" t="inlineStr">
+        <is>
+          <t>Monitoring Console</t>
+        </is>
+      </c>
+      <c r="D38" s="17" t="inlineStr">
+        <is>
+          <t>a001</t>
+        </is>
+      </c>
+      <c r="E38" s="17" t="inlineStr">
+        <is>
+          <t>ESB Platform</t>
+        </is>
+      </c>
+      <c r="F38" s="23" t="inlineStr">
         <is>
           <t>AssociationRelationship</t>
         </is>
       </c>
-      <c r="G2" s="16" t="inlineStr"/>
-      <c r="H2" s="16" t="n"/>
-      <c r="I2" s="16" t="n"/>
-    </row>
-    <row r="3">
-      <c r="A3" s="16" t="inlineStr"/>
-      <c r="B3" s="16" t="inlineStr">
-        <is>
-          <t>&lt;App Component ID&gt;</t>
-        </is>
-      </c>
-      <c r="C3" s="16" t="inlineStr">
-        <is>
-          <t>Order Management System</t>
-        </is>
-      </c>
-      <c r="D3" s="17" t="inlineStr">
-        <is>
-          <t>&lt;Business Service ID&gt;</t>
-        </is>
-      </c>
-      <c r="E3" s="17" t="inlineStr">
-        <is>
-          <t>Order Management</t>
-        </is>
-      </c>
-      <c r="F3" s="16" t="inlineStr">
+      <c r="G38" s="23" t="inlineStr"/>
+      <c r="H38" s="23" t="inlineStr"/>
+      <c r="I38" s="23" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="23" t="inlineStr"/>
+      <c r="B39" s="23" t="inlineStr">
+        <is>
+          <t>a011</t>
+        </is>
+      </c>
+      <c r="C39" s="23" t="inlineStr">
+        <is>
+          <t>Integration Schema</t>
+        </is>
+      </c>
+      <c r="D39" s="17" t="inlineStr">
+        <is>
+          <t>a007</t>
+        </is>
+      </c>
+      <c r="E39" s="17" t="inlineStr">
+        <is>
+          <t>Message Routing Svc</t>
+        </is>
+      </c>
+      <c r="F39" s="23" t="inlineStr">
+        <is>
+          <t>AssociationRelationship</t>
+        </is>
+      </c>
+      <c r="G39" s="23" t="inlineStr"/>
+      <c r="H39" s="23" t="inlineStr"/>
+      <c r="I39" s="23" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="23" t="inlineStr"/>
+      <c r="B40" s="23" t="inlineStr">
+        <is>
+          <t>a012</t>
+        </is>
+      </c>
+      <c r="C40" s="23" t="inlineStr">
+        <is>
+          <t>API Specification</t>
+        </is>
+      </c>
+      <c r="D40" s="17" t="inlineStr">
+        <is>
+          <t>a002</t>
+        </is>
+      </c>
+      <c r="E40" s="17" t="inlineStr">
+        <is>
+          <t>API Gateway</t>
+        </is>
+      </c>
+      <c r="F40" s="23" t="inlineStr">
+        <is>
+          <t>AssociationRelationship</t>
+        </is>
+      </c>
+      <c r="G40" s="23" t="inlineStr"/>
+      <c r="H40" s="23" t="inlineStr"/>
+      <c r="I40" s="23" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="23" t="inlineStr"/>
+      <c r="B41" s="23" t="inlineStr">
+        <is>
+          <t>a013</t>
+        </is>
+      </c>
+      <c r="C41" s="23" t="inlineStr">
+        <is>
+          <t>SLA Definition</t>
+        </is>
+      </c>
+      <c r="D41" s="17" t="inlineStr">
+        <is>
+          <t>a005</t>
+        </is>
+      </c>
+      <c r="E41" s="17" t="inlineStr">
+        <is>
+          <t>Monitoring Console</t>
+        </is>
+      </c>
+      <c r="F41" s="23" t="inlineStr">
+        <is>
+          <t>AssociationRelationship</t>
+        </is>
+      </c>
+      <c r="G41" s="23" t="inlineStr"/>
+      <c r="H41" s="23" t="inlineStr"/>
+      <c r="I41" s="23" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="23" t="inlineStr"/>
+      <c r="B42" s="23" t="inlineStr">
+        <is>
+          <t>t001</t>
+        </is>
+      </c>
+      <c r="C42" s="23" t="inlineStr">
+        <is>
+          <t>Integration Server</t>
+        </is>
+      </c>
+      <c r="D42" s="17" t="inlineStr">
+        <is>
+          <t>a001</t>
+        </is>
+      </c>
+      <c r="E42" s="17" t="inlineStr">
+        <is>
+          <t>ESB Platform</t>
+        </is>
+      </c>
+      <c r="F42" s="23" t="inlineStr">
+        <is>
+          <t>AssignmentRelationship</t>
+        </is>
+      </c>
+      <c r="G42" s="23" t="inlineStr"/>
+      <c r="H42" s="23" t="inlineStr"/>
+      <c r="I42" s="23" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="23" t="inlineStr"/>
+      <c r="B43" s="23" t="inlineStr">
+        <is>
+          <t>t002</t>
+        </is>
+      </c>
+      <c r="C43" s="23" t="inlineStr">
+        <is>
+          <t>Message Queue Server</t>
+        </is>
+      </c>
+      <c r="D43" s="17" t="inlineStr">
+        <is>
+          <t>a003</t>
+        </is>
+      </c>
+      <c r="E43" s="17" t="inlineStr">
+        <is>
+          <t>Message Broker</t>
+        </is>
+      </c>
+      <c r="F43" s="23" t="inlineStr">
+        <is>
+          <t>AssignmentRelationship</t>
+        </is>
+      </c>
+      <c r="G43" s="23" t="inlineStr"/>
+      <c r="H43" s="23" t="inlineStr"/>
+      <c r="I43" s="23" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="23" t="inlineStr"/>
+      <c r="B44" s="23" t="inlineStr">
+        <is>
+          <t>t003</t>
+        </is>
+      </c>
+      <c r="C44" s="23" t="inlineStr">
+        <is>
+          <t>API Gateway Server</t>
+        </is>
+      </c>
+      <c r="D44" s="17" t="inlineStr">
+        <is>
+          <t>a002</t>
+        </is>
+      </c>
+      <c r="E44" s="17" t="inlineStr">
+        <is>
+          <t>API Gateway</t>
+        </is>
+      </c>
+      <c r="F44" s="23" t="inlineStr">
+        <is>
+          <t>AssignmentRelationship</t>
+        </is>
+      </c>
+      <c r="G44" s="23" t="inlineStr"/>
+      <c r="H44" s="23" t="inlineStr"/>
+      <c r="I44" s="23" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="23" t="inlineStr"/>
+      <c r="B45" s="23" t="inlineStr">
+        <is>
+          <t>t004</t>
+        </is>
+      </c>
+      <c r="C45" s="23" t="inlineStr">
+        <is>
+          <t>ESB Software Package</t>
+        </is>
+      </c>
+      <c r="D45" s="17" t="inlineStr">
+        <is>
+          <t>a001</t>
+        </is>
+      </c>
+      <c r="E45" s="17" t="inlineStr">
+        <is>
+          <t>ESB Platform</t>
+        </is>
+      </c>
+      <c r="F45" s="23" t="inlineStr">
         <is>
           <t>RealizationRelationship</t>
         </is>
       </c>
-      <c r="G3" s="16" t="inlineStr"/>
-      <c r="H3" s="16" t="n"/>
-      <c r="I3" s="16" t="n"/>
-    </row>
-    <row r="4">
-      <c r="A4" s="16" t="inlineStr"/>
-      <c r="B4" s="16" t="inlineStr">
-        <is>
-          <t>&lt;App Component ID&gt;</t>
-        </is>
-      </c>
-      <c r="C4" s="16" t="inlineStr">
-        <is>
-          <t>CRM System</t>
-        </is>
-      </c>
-      <c r="D4" s="17" t="inlineStr">
-        <is>
-          <t>&lt;Business Actor ID&gt;</t>
-        </is>
-      </c>
-      <c r="E4" s="17" t="inlineStr">
-        <is>
-          <t>Customer</t>
-        </is>
-      </c>
-      <c r="F4" s="16" t="inlineStr">
+      <c r="G45" s="23" t="inlineStr"/>
+      <c r="H45" s="23" t="inlineStr"/>
+      <c r="I45" s="23" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="23" t="inlineStr"/>
+      <c r="B46" s="23" t="inlineStr">
+        <is>
+          <t>t005</t>
+        </is>
+      </c>
+      <c r="C46" s="23" t="inlineStr">
+        <is>
+          <t>Container Platform</t>
+        </is>
+      </c>
+      <c r="D46" s="17" t="inlineStr">
+        <is>
+          <t>a001</t>
+        </is>
+      </c>
+      <c r="E46" s="17" t="inlineStr">
+        <is>
+          <t>ESB Platform</t>
+        </is>
+      </c>
+      <c r="F46" s="23" t="inlineStr">
+        <is>
+          <t>AssignmentRelationship</t>
+        </is>
+      </c>
+      <c r="G46" s="23" t="inlineStr"/>
+      <c r="H46" s="23" t="inlineStr"/>
+      <c r="I46" s="23" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="23" t="inlineStr"/>
+      <c r="B47" s="23" t="inlineStr">
+        <is>
+          <t>t006</t>
+        </is>
+      </c>
+      <c r="C47" s="23" t="inlineStr">
+        <is>
+          <t>Operating System</t>
+        </is>
+      </c>
+      <c r="D47" s="17" t="inlineStr">
+        <is>
+          <t>t001</t>
+        </is>
+      </c>
+      <c r="E47" s="17" t="inlineStr">
+        <is>
+          <t>Integration Server</t>
+        </is>
+      </c>
+      <c r="F47" s="23" t="inlineStr">
+        <is>
+          <t>AssignmentRelationship</t>
+        </is>
+      </c>
+      <c r="G47" s="23" t="inlineStr"/>
+      <c r="H47" s="23" t="inlineStr"/>
+      <c r="I47" s="23" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="23" t="inlineStr"/>
+      <c r="B48" s="23" t="inlineStr">
+        <is>
+          <t>t006</t>
+        </is>
+      </c>
+      <c r="C48" s="23" t="inlineStr">
+        <is>
+          <t>Operating System</t>
+        </is>
+      </c>
+      <c r="D48" s="17" t="inlineStr">
+        <is>
+          <t>t002</t>
+        </is>
+      </c>
+      <c r="E48" s="17" t="inlineStr">
+        <is>
+          <t>Message Queue Server</t>
+        </is>
+      </c>
+      <c r="F48" s="23" t="inlineStr">
+        <is>
+          <t>AssignmentRelationship</t>
+        </is>
+      </c>
+      <c r="G48" s="23" t="inlineStr"/>
+      <c r="H48" s="23" t="inlineStr"/>
+      <c r="I48" s="23" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="23" t="inlineStr"/>
+      <c r="B49" s="23" t="inlineStr">
+        <is>
+          <t>t007</t>
+        </is>
+      </c>
+      <c r="C49" s="23" t="inlineStr">
+        <is>
+          <t>Municipal Network</t>
+        </is>
+      </c>
+      <c r="D49" s="17" t="inlineStr">
+        <is>
+          <t>t001</t>
+        </is>
+      </c>
+      <c r="E49" s="17" t="inlineStr">
+        <is>
+          <t>Integration Server</t>
+        </is>
+      </c>
+      <c r="F49" s="23" t="inlineStr">
         <is>
           <t>ServingRelationship</t>
         </is>
       </c>
-      <c r="G4" s="16" t="inlineStr"/>
-      <c r="H4" s="16" t="n"/>
-      <c r="I4" s="16" t="n"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="16" t="inlineStr"/>
-      <c r="B5" s="16" t="inlineStr">
-        <is>
-          <t>&lt;Tech Node ID&gt;</t>
-        </is>
-      </c>
-      <c r="C5" s="16" t="inlineStr">
-        <is>
-          <t>Application Server</t>
-        </is>
-      </c>
-      <c r="D5" s="17" t="inlineStr">
-        <is>
-          <t>&lt;App Component ID&gt;</t>
-        </is>
-      </c>
-      <c r="E5" s="17" t="inlineStr">
-        <is>
-          <t>Order Management System</t>
-        </is>
-      </c>
-      <c r="F5" s="16" t="inlineStr">
-        <is>
-          <t>AssignmentRelationship</t>
-        </is>
-      </c>
-      <c r="G5" s="16" t="inlineStr"/>
-      <c r="H5" s="16" t="n"/>
-      <c r="I5" s="16" t="n"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="16" t="inlineStr"/>
-      <c r="B6" s="16" t="inlineStr">
-        <is>
-          <t>&lt;Tech Node ID&gt;</t>
-        </is>
-      </c>
-      <c r="C6" s="16" t="inlineStr">
-        <is>
-          <t>Database Server</t>
-        </is>
-      </c>
-      <c r="D6" s="17" t="inlineStr">
-        <is>
-          <t>&lt;App Component ID&gt;</t>
-        </is>
-      </c>
-      <c r="E6" s="17" t="inlineStr">
-        <is>
-          <t>Order Management System</t>
-        </is>
-      </c>
-      <c r="F6" s="16" t="inlineStr">
-        <is>
-          <t>AssignmentRelationship</t>
-        </is>
-      </c>
-      <c r="G6" s="16" t="inlineStr"/>
-      <c r="H6" s="16" t="n"/>
-      <c r="I6" s="16" t="n"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="16" t="n"/>
-      <c r="B7" s="16" t="n"/>
-      <c r="C7" s="16" t="n"/>
-      <c r="D7" s="17" t="n"/>
-      <c r="E7" s="17" t="n"/>
-      <c r="F7" s="16" t="n"/>
-      <c r="G7" s="16" t="n"/>
-      <c r="H7" s="16" t="n"/>
-      <c r="I7" s="16" t="n"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="16" t="n"/>
-      <c r="B8" s="16" t="n"/>
-      <c r="C8" s="16" t="n"/>
-      <c r="D8" s="17" t="n"/>
-      <c r="E8" s="17" t="n"/>
-      <c r="F8" s="16" t="n"/>
-      <c r="G8" s="16" t="n"/>
-      <c r="H8" s="16" t="n"/>
-      <c r="I8" s="16" t="n"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="16" t="n"/>
-      <c r="B9" s="16" t="n"/>
-      <c r="C9" s="16" t="n"/>
-      <c r="D9" s="17" t="n"/>
-      <c r="E9" s="17" t="n"/>
-      <c r="F9" s="16" t="n"/>
-      <c r="G9" s="16" t="n"/>
-      <c r="H9" s="16" t="n"/>
-      <c r="I9" s="16" t="n"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="16" t="n"/>
-      <c r="B10" s="16" t="n"/>
-      <c r="C10" s="16" t="n"/>
-      <c r="D10" s="17" t="n"/>
-      <c r="E10" s="17" t="n"/>
-      <c r="F10" s="16" t="n"/>
-      <c r="G10" s="16" t="n"/>
-      <c r="H10" s="16" t="n"/>
-      <c r="I10" s="16" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="16" t="n"/>
-      <c r="B11" s="16" t="n"/>
-      <c r="C11" s="16" t="n"/>
-      <c r="D11" s="17" t="n"/>
-      <c r="E11" s="17" t="n"/>
-      <c r="F11" s="16" t="n"/>
-      <c r="G11" s="16" t="n"/>
-      <c r="H11" s="16" t="n"/>
-      <c r="I11" s="16" t="n"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="16" t="n"/>
-      <c r="B12" s="16" t="n"/>
-      <c r="C12" s="16" t="n"/>
-      <c r="D12" s="17" t="n"/>
-      <c r="E12" s="17" t="n"/>
-      <c r="F12" s="16" t="n"/>
-      <c r="G12" s="16" t="n"/>
-      <c r="H12" s="16" t="n"/>
-      <c r="I12" s="16" t="n"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="16" t="n"/>
-      <c r="B13" s="16" t="n"/>
-      <c r="C13" s="16" t="n"/>
-      <c r="D13" s="17" t="n"/>
-      <c r="E13" s="17" t="n"/>
-      <c r="F13" s="16" t="n"/>
-      <c r="G13" s="16" t="n"/>
-      <c r="H13" s="16" t="n"/>
-      <c r="I13" s="16" t="n"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="16" t="n"/>
-      <c r="B14" s="16" t="n"/>
-      <c r="C14" s="16" t="n"/>
-      <c r="D14" s="17" t="n"/>
-      <c r="E14" s="17" t="n"/>
-      <c r="F14" s="16" t="n"/>
-      <c r="G14" s="16" t="n"/>
-      <c r="H14" s="16" t="n"/>
-      <c r="I14" s="16" t="n"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="16" t="n"/>
-      <c r="B15" s="16" t="n"/>
-      <c r="C15" s="16" t="n"/>
-      <c r="D15" s="17" t="n"/>
-      <c r="E15" s="17" t="n"/>
-      <c r="F15" s="16" t="n"/>
-      <c r="G15" s="16" t="n"/>
-      <c r="H15" s="16" t="n"/>
-      <c r="I15" s="16" t="n"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="16" t="n"/>
-      <c r="B16" s="16" t="n"/>
-      <c r="C16" s="16" t="n"/>
-      <c r="D16" s="17" t="n"/>
-      <c r="E16" s="17" t="n"/>
-      <c r="F16" s="16" t="n"/>
-      <c r="G16" s="16" t="n"/>
-      <c r="H16" s="16" t="n"/>
-      <c r="I16" s="16" t="n"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="16" t="n"/>
-      <c r="B17" s="16" t="n"/>
-      <c r="C17" s="16" t="n"/>
-      <c r="D17" s="17" t="n"/>
-      <c r="E17" s="17" t="n"/>
-      <c r="F17" s="16" t="n"/>
-      <c r="G17" s="16" t="n"/>
-      <c r="H17" s="16" t="n"/>
-      <c r="I17" s="16" t="n"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="16" t="n"/>
-      <c r="B18" s="16" t="n"/>
-      <c r="C18" s="16" t="n"/>
-      <c r="D18" s="17" t="n"/>
-      <c r="E18" s="17" t="n"/>
-      <c r="F18" s="16" t="n"/>
-      <c r="G18" s="16" t="n"/>
-      <c r="H18" s="16" t="n"/>
-      <c r="I18" s="16" t="n"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="16" t="n"/>
-      <c r="B19" s="16" t="n"/>
-      <c r="C19" s="16" t="n"/>
-      <c r="D19" s="17" t="n"/>
-      <c r="E19" s="17" t="n"/>
-      <c r="F19" s="16" t="n"/>
-      <c r="G19" s="16" t="n"/>
-      <c r="H19" s="16" t="n"/>
-      <c r="I19" s="16" t="n"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="16" t="n"/>
-      <c r="B20" s="16" t="n"/>
-      <c r="C20" s="16" t="n"/>
-      <c r="D20" s="17" t="n"/>
-      <c r="E20" s="17" t="n"/>
-      <c r="F20" s="16" t="n"/>
-      <c r="G20" s="16" t="n"/>
-      <c r="H20" s="16" t="n"/>
-      <c r="I20" s="16" t="n"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="16" t="n"/>
-      <c r="B21" s="16" t="n"/>
-      <c r="C21" s="16" t="n"/>
-      <c r="D21" s="17" t="n"/>
-      <c r="E21" s="17" t="n"/>
-      <c r="F21" s="16" t="n"/>
-      <c r="G21" s="16" t="n"/>
-      <c r="H21" s="16" t="n"/>
-      <c r="I21" s="16" t="n"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="16" t="n"/>
-      <c r="B22" s="16" t="n"/>
-      <c r="C22" s="16" t="n"/>
-      <c r="D22" s="17" t="n"/>
-      <c r="E22" s="17" t="n"/>
-      <c r="F22" s="16" t="n"/>
-      <c r="G22" s="16" t="n"/>
-      <c r="H22" s="16" t="n"/>
-      <c r="I22" s="16" t="n"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="16" t="n"/>
-      <c r="B23" s="16" t="n"/>
-      <c r="C23" s="16" t="n"/>
-      <c r="D23" s="17" t="n"/>
-      <c r="E23" s="17" t="n"/>
-      <c r="F23" s="16" t="n"/>
-      <c r="G23" s="16" t="n"/>
-      <c r="H23" s="16" t="n"/>
-      <c r="I23" s="16" t="n"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="16" t="n"/>
-      <c r="B24" s="16" t="n"/>
-      <c r="C24" s="16" t="n"/>
-      <c r="D24" s="17" t="n"/>
-      <c r="E24" s="17" t="n"/>
-      <c r="F24" s="16" t="n"/>
-      <c r="G24" s="16" t="n"/>
-      <c r="H24" s="16" t="n"/>
-      <c r="I24" s="16" t="n"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="16" t="n"/>
-      <c r="B25" s="16" t="n"/>
-      <c r="C25" s="16" t="n"/>
-      <c r="D25" s="17" t="n"/>
-      <c r="E25" s="17" t="n"/>
-      <c r="F25" s="16" t="n"/>
-      <c r="G25" s="16" t="n"/>
-      <c r="H25" s="16" t="n"/>
-      <c r="I25" s="16" t="n"/>
-    </row>
-    <row r="26">
-      <c r="A26" s="16" t="n"/>
-      <c r="B26" s="16" t="n"/>
-      <c r="C26" s="16" t="n"/>
-      <c r="D26" s="17" t="n"/>
-      <c r="E26" s="17" t="n"/>
-      <c r="F26" s="16" t="n"/>
-      <c r="G26" s="16" t="n"/>
-      <c r="H26" s="16" t="n"/>
-      <c r="I26" s="16" t="n"/>
+      <c r="G49" s="23" t="inlineStr"/>
+      <c r="H49" s="23" t="inlineStr"/>
+      <c r="I49" s="23" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="23" t="inlineStr"/>
+      <c r="B50" s="23" t="inlineStr">
+        <is>
+          <t>t007</t>
+        </is>
+      </c>
+      <c r="C50" s="23" t="inlineStr">
+        <is>
+          <t>Municipal Network</t>
+        </is>
+      </c>
+      <c r="D50" s="17" t="inlineStr">
+        <is>
+          <t>t002</t>
+        </is>
+      </c>
+      <c r="E50" s="17" t="inlineStr">
+        <is>
+          <t>Message Queue Server</t>
+        </is>
+      </c>
+      <c r="F50" s="23" t="inlineStr">
+        <is>
+          <t>ServingRelationship</t>
+        </is>
+      </c>
+      <c r="G50" s="23" t="inlineStr"/>
+      <c r="H50" s="23" t="inlineStr"/>
+      <c r="I50" s="23" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="23" t="inlineStr"/>
+      <c r="B51" s="23" t="inlineStr">
+        <is>
+          <t>t008</t>
+        </is>
+      </c>
+      <c r="C51" s="23" t="inlineStr">
+        <is>
+          <t>DMZ</t>
+        </is>
+      </c>
+      <c r="D51" s="17" t="inlineStr">
+        <is>
+          <t>t003</t>
+        </is>
+      </c>
+      <c r="E51" s="17" t="inlineStr">
+        <is>
+          <t>API Gateway Server</t>
+        </is>
+      </c>
+      <c r="F51" s="23" t="inlineStr">
+        <is>
+          <t>ServingRelationship</t>
+        </is>
+      </c>
+      <c r="G51" s="23" t="inlineStr"/>
+      <c r="H51" s="23" t="inlineStr"/>
+      <c r="I51" s="23" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="23" t="inlineStr"/>
+      <c r="B52" s="23" t="inlineStr">
+        <is>
+          <t>t009</t>
+        </is>
+      </c>
+      <c r="C52" s="23" t="inlineStr">
+        <is>
+          <t>Deployment Package</t>
+        </is>
+      </c>
+      <c r="D52" s="17" t="inlineStr">
+        <is>
+          <t>a001</t>
+        </is>
+      </c>
+      <c r="E52" s="17" t="inlineStr">
+        <is>
+          <t>ESB Platform</t>
+        </is>
+      </c>
+      <c r="F52" s="23" t="inlineStr">
+        <is>
+          <t>AssociationRelationship</t>
+        </is>
+      </c>
+      <c r="G52" s="23" t="inlineStr"/>
+      <c r="H52" s="23" t="inlineStr"/>
+      <c r="I52" s="23" t="inlineStr"/>
     </row>
   </sheetData>
   <dataValidations count="2">
@@ -2586,15 +4539,15 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="18" t="inlineStr"/>
-      <c r="B2" s="18" t="inlineStr">
+      <c r="A2" s="24" t="inlineStr"/>
+      <c r="B2" s="24" t="inlineStr">
         <is>
           <t>Full Architecture View</t>
         </is>
       </c>
-      <c r="C2" s="18" t="inlineStr">
-        <is>
-          <t>Complete view of all architecture layers</t>
+      <c r="C2" s="24" t="inlineStr">
+        <is>
+          <t>Complete layered overview of the municipal ESB tender — Business, Application and Technology</t>
         </is>
       </c>
       <c r="D2" s="19" t="inlineStr"/>
@@ -2603,70 +4556,70 @@
           <t>ALL</t>
         </is>
       </c>
-      <c r="F2" s="18" t="inlineStr">
+      <c r="F2" s="24" t="inlineStr">
         <is>
           <t>ArchiMate View</t>
         </is>
       </c>
-      <c r="G2" s="18" t="inlineStr">
+      <c r="G2" s="24" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="18" t="inlineStr"/>
-      <c r="B3" s="18" t="inlineStr">
-        <is>
-          <t>Business Layer</t>
-        </is>
-      </c>
-      <c r="C3" s="18" t="inlineStr">
-        <is>
-          <t>Business processes, actors, and services only</t>
+      <c r="A3" s="24" t="inlineStr"/>
+      <c r="B3" s="24" t="inlineStr">
+        <is>
+          <t>Tender Process</t>
+        </is>
+      </c>
+      <c r="C3" s="24" t="inlineStr">
+        <is>
+          <t>EU procurement lifecycle from needs assessment through contract award and implementation</t>
         </is>
       </c>
       <c r="D3" s="19" t="inlineStr"/>
       <c r="E3" s="19" t="inlineStr">
         <is>
-          <t>&lt;comma-sep business IDs&gt;</t>
-        </is>
-      </c>
-      <c r="F3" s="18" t="inlineStr">
+          <t>b001,b002,b003,b004,b005,b006,b007,b008,b009,b010,b011,b012,b013,b014,b015,b016,b017,b018,b019,b020</t>
+        </is>
+      </c>
+      <c r="F3" s="24" t="inlineStr">
         <is>
           <t>ArchiMate View</t>
         </is>
       </c>
-      <c r="G3" s="18" t="inlineStr">
+      <c r="G3" s="24" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="18" t="inlineStr"/>
-      <c r="B4" s="18" t="inlineStr">
-        <is>
-          <t>Application Architecture</t>
-        </is>
-      </c>
-      <c r="C4" s="18" t="inlineStr">
-        <is>
-          <t>Application components and their connections</t>
+      <c r="A4" s="24" t="inlineStr"/>
+      <c r="B4" s="24" t="inlineStr">
+        <is>
+          <t>ESB Solution Architecture</t>
+        </is>
+      </c>
+      <c r="C4" s="24" t="inlineStr">
+        <is>
+          <t>Application components, services, data objects and technology infrastructure for the ESB</t>
         </is>
       </c>
       <c r="D4" s="19" t="inlineStr"/>
       <c r="E4" s="19" t="inlineStr">
         <is>
-          <t>&lt;comma-sep app IDs&gt;</t>
-        </is>
-      </c>
-      <c r="F4" s="18" t="inlineStr">
+          <t>a001,a002,a003,a004,a005,a006,a007,a008,a009,a010,a011,a012,a013,t001,t002,t003,t004,t005,t006,t007,t008,t009</t>
+        </is>
+      </c>
+      <c r="F4" s="24" t="inlineStr">
         <is>
           <t>ArchiMate View</t>
         </is>
       </c>
-      <c r="G4" s="18" t="inlineStr">
+      <c r="G4" s="24" t="inlineStr">
         <is>
           <t>No</t>
         </is>

</xml_diff>